<commit_message>
feat: implement KRX+NXT integrated data fetching for trading signals
- Add _AL suffix to stock codes for integrated market data retrieval
- Fix Trading_Signal_System.py to use KRX+NXT combined data instead of KRX-only
- Update chart data fetching to use integrated ticker format (e.g., 005930_AL)
- Resolve price discrepancy between integrated chart and trading signals
- Add comprehensive documentation and monitoring guides
- Update trading signals with integrated market data
- Add batch files for automated system execution
</commit_message>
<xml_diff>
--- a/trading_signals.xlsx
+++ b/trading_signals.xlsx
@@ -457,7 +457,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AH67"/>
+  <dimension ref="A1:AH68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -664,7 +664,7 @@
       </c>
       <c r="AH1" s="4" t="inlineStr">
         <is>
-          <t>최종 업데이트: 2025-10-14 00:23:08</t>
+          <t>최종 업데이트: 2025-10-16 03:37:24</t>
         </is>
       </c>
     </row>
@@ -691,45 +691,45 @@
       </c>
       <c r="E2" s="6" t="inlineStr">
         <is>
-          <t>1차 매수선까지 41.9%</t>
+          <t>1차 매수선까지 41.4%</t>
         </is>
       </c>
       <c r="F2" s="7" t="n">
-        <v>93300</v>
+        <v>95500</v>
       </c>
       <c r="G2" s="7" t="n">
-        <v>90700</v>
+        <v>91400</v>
       </c>
       <c r="H2" s="7" t="n">
-        <v>93400</v>
+        <v>95600</v>
       </c>
       <c r="I2" s="7" t="n">
-        <v>82050</v>
+        <v>84270</v>
       </c>
       <c r="J2" s="7" t="n">
-        <v>65640</v>
+        <v>67416</v>
       </c>
       <c r="K2" s="7" t="n">
-        <v>65740</v>
+        <v>67516</v>
       </c>
       <c r="L2" s="8" t="n">
-        <v>0.4192272588986918</v>
+        <v>0.4144795307778897</v>
       </c>
       <c r="M2" s="9" t="inlineStr"/>
       <c r="N2" s="9" t="inlineStr"/>
       <c r="O2" s="7" t="n">
-        <v>59166</v>
+        <v>60764.4</v>
       </c>
       <c r="P2" s="8" t="n">
-        <v>0.5769191765541019</v>
+        <v>0.5716439230865441</v>
       </c>
       <c r="Q2" s="9" t="inlineStr"/>
       <c r="R2" s="9" t="inlineStr"/>
       <c r="S2" s="7" t="n">
-        <v>53249.4</v>
+        <v>54687.96</v>
       </c>
       <c r="T2" s="8" t="n">
-        <v>0.7521324183934468</v>
+        <v>0.7462710256517157</v>
       </c>
       <c r="U2" s="9" t="inlineStr"/>
       <c r="V2" s="9" t="inlineStr"/>
@@ -743,7 +743,7 @@
       <c r="AD2" s="9" t="inlineStr"/>
       <c r="AE2" s="10" t="inlineStr">
         <is>
-          <t>2025-10-14 00:22:45</t>
+          <t>2025-10-16 03:37:02</t>
         </is>
       </c>
       <c r="AF2" s="11" t="n">
@@ -775,45 +775,45 @@
       </c>
       <c r="E3" s="6" t="inlineStr">
         <is>
-          <t>1차 매수선까지 47.9%</t>
+          <t>1차 매수선까지 46.3%</t>
         </is>
       </c>
       <c r="F3" s="7" t="n">
-        <v>415000</v>
+        <v>425500</v>
       </c>
       <c r="G3" s="7" t="n">
-        <v>403000</v>
+        <v>404500</v>
       </c>
       <c r="H3" s="7" t="n">
-        <v>415500</v>
+        <v>425500</v>
       </c>
       <c r="I3" s="7" t="n">
-        <v>350175</v>
+        <v>363050</v>
       </c>
       <c r="J3" s="7" t="n">
-        <v>280140</v>
+        <v>290440</v>
       </c>
       <c r="K3" s="7" t="n">
-        <v>280640</v>
+        <v>290940</v>
       </c>
       <c r="L3" s="8" t="n">
-        <v>0.4787628278221209</v>
+        <v>0.4625008592837011</v>
       </c>
       <c r="M3" s="9" t="inlineStr"/>
       <c r="N3" s="9" t="inlineStr"/>
       <c r="O3" s="7" t="n">
-        <v>252576</v>
+        <v>261846</v>
       </c>
       <c r="P3" s="8" t="n">
-        <v>0.6430698086912454</v>
+        <v>0.6250009547596679</v>
       </c>
       <c r="Q3" s="9" t="inlineStr"/>
       <c r="R3" s="9" t="inlineStr"/>
       <c r="S3" s="7" t="n">
-        <v>227318.4</v>
+        <v>235661.4</v>
       </c>
       <c r="T3" s="8" t="n">
-        <v>0.8256331207680505</v>
+        <v>0.8055566163996311</v>
       </c>
       <c r="U3" s="9" t="inlineStr"/>
       <c r="V3" s="9" t="inlineStr"/>
@@ -827,7 +827,7 @@
       <c r="AD3" s="9" t="inlineStr"/>
       <c r="AE3" s="10" t="inlineStr">
         <is>
-          <t>2025-10-14 00:22:46</t>
+          <t>2025-10-16 03:37:02</t>
         </is>
       </c>
       <c r="AF3" s="11" t="n">
@@ -859,45 +859,45 @@
       </c>
       <c r="E4" s="6" t="inlineStr">
         <is>
-          <t>1차 매수선까지 51.6%</t>
+          <t>1차 매수선까지 60.3%</t>
         </is>
       </c>
       <c r="F4" s="7" t="n">
-        <v>77600</v>
+        <v>84300</v>
       </c>
       <c r="G4" s="7" t="n">
-        <v>73400</v>
+        <v>75200</v>
       </c>
       <c r="H4" s="7" t="n">
-        <v>78500</v>
+        <v>84900</v>
       </c>
       <c r="I4" s="7" t="n">
-        <v>63860</v>
+        <v>65610</v>
       </c>
       <c r="J4" s="7" t="n">
-        <v>51088</v>
+        <v>52488</v>
       </c>
       <c r="K4" s="7" t="n">
-        <v>51188</v>
+        <v>52588</v>
       </c>
       <c r="L4" s="8" t="n">
-        <v>0.5159803078846604</v>
+        <v>0.603027306609873</v>
       </c>
       <c r="M4" s="9" t="inlineStr"/>
       <c r="N4" s="9" t="inlineStr"/>
       <c r="O4" s="7" t="n">
-        <v>46069.2</v>
+        <v>47329.2</v>
       </c>
       <c r="P4" s="8" t="n">
-        <v>0.6844225643162892</v>
+        <v>0.7811414517887476</v>
       </c>
       <c r="Q4" s="9" t="inlineStr"/>
       <c r="R4" s="9" t="inlineStr"/>
       <c r="S4" s="7" t="n">
-        <v>41462.28000000001</v>
+        <v>42596.28000000001</v>
       </c>
       <c r="T4" s="8" t="n">
-        <v>0.871580627018099</v>
+        <v>0.9790460575430529</v>
       </c>
       <c r="U4" s="9" t="inlineStr"/>
       <c r="V4" s="9" t="inlineStr"/>
@@ -911,7 +911,7 @@
       <c r="AD4" s="9" t="inlineStr"/>
       <c r="AE4" s="10" t="inlineStr">
         <is>
-          <t>2025-10-14 00:22:46</t>
+          <t>2025-10-16 03:37:03</t>
         </is>
       </c>
       <c r="AF4" s="11" t="n">
@@ -943,45 +943,45 @@
       </c>
       <c r="E5" s="6" t="inlineStr">
         <is>
-          <t>1차 매수선까지 33.8%</t>
+          <t>1차 매수선까지 30.5%</t>
         </is>
       </c>
       <c r="F5" s="7" t="n">
-        <v>262500</v>
+        <v>259000</v>
       </c>
       <c r="G5" s="7" t="n">
-        <v>258000</v>
+        <v>255000</v>
       </c>
       <c r="H5" s="7" t="n">
-        <v>266500</v>
+        <v>264000</v>
       </c>
       <c r="I5" s="7" t="n">
-        <v>244525</v>
+        <v>247550</v>
       </c>
       <c r="J5" s="7" t="n">
-        <v>195620</v>
+        <v>198040</v>
       </c>
       <c r="K5" s="7" t="n">
-        <v>196120</v>
+        <v>198540</v>
       </c>
       <c r="L5" s="8" t="n">
-        <v>0.3384662451560269</v>
+        <v>0.3045230180316309</v>
       </c>
       <c r="M5" s="9" t="inlineStr"/>
       <c r="N5" s="9" t="inlineStr"/>
       <c r="O5" s="7" t="n">
-        <v>176508</v>
+        <v>178686</v>
       </c>
       <c r="P5" s="8" t="n">
-        <v>0.4871847168400299</v>
+        <v>0.4494700200351455</v>
       </c>
       <c r="Q5" s="9" t="inlineStr"/>
       <c r="R5" s="9" t="inlineStr"/>
       <c r="S5" s="7" t="n">
-        <v>158857.2</v>
+        <v>160817.4</v>
       </c>
       <c r="T5" s="8" t="n">
-        <v>0.6524274631555886</v>
+        <v>0.610522244483495</v>
       </c>
       <c r="U5" s="9" t="inlineStr"/>
       <c r="V5" s="9" t="inlineStr"/>
@@ -995,7 +995,7 @@
       <c r="AD5" s="9" t="inlineStr"/>
       <c r="AE5" s="10" t="inlineStr">
         <is>
-          <t>2025-10-14 00:22:46</t>
+          <t>2025-10-16 03:37:03</t>
         </is>
       </c>
       <c r="AF5" s="11" t="n">
@@ -1027,45 +1027,45 @@
       </c>
       <c r="E6" s="6" t="inlineStr">
         <is>
-          <t>1차 매수선까지 66.9%</t>
+          <t>1차 매수선까지 78.3%</t>
         </is>
       </c>
       <c r="F6" s="7" t="n">
-        <v>128000</v>
+        <v>144000</v>
       </c>
       <c r="G6" s="7" t="n">
-        <v>114000</v>
+        <v>125700</v>
       </c>
       <c r="H6" s="7" t="n">
-        <v>129800</v>
+        <v>144600</v>
       </c>
       <c r="I6" s="7" t="n">
-        <v>95755</v>
+        <v>100830</v>
       </c>
       <c r="J6" s="7" t="n">
-        <v>76604</v>
+        <v>80664</v>
       </c>
       <c r="K6" s="7" t="n">
-        <v>76704</v>
+        <v>80764</v>
       </c>
       <c r="L6" s="8" t="n">
-        <v>0.6687526074259492</v>
+        <v>0.7829726115596057</v>
       </c>
       <c r="M6" s="9" t="inlineStr"/>
       <c r="N6" s="9" t="inlineStr"/>
       <c r="O6" s="7" t="n">
-        <v>69033.60000000001</v>
+        <v>72687.60000000001</v>
       </c>
       <c r="P6" s="8" t="n">
-        <v>0.8541695638066099</v>
+        <v>0.9810806795106728</v>
       </c>
       <c r="Q6" s="9" t="inlineStr"/>
       <c r="R6" s="9" t="inlineStr"/>
       <c r="S6" s="7" t="n">
-        <v>62130.24000000001</v>
+        <v>65418.84</v>
       </c>
       <c r="T6" s="8" t="n">
-        <v>1.060188404229567</v>
+        <v>1.201200755011859</v>
       </c>
       <c r="U6" s="9" t="inlineStr"/>
       <c r="V6" s="9" t="inlineStr"/>
@@ -1079,7 +1079,7 @@
       <c r="AD6" s="9" t="inlineStr"/>
       <c r="AE6" s="10" t="inlineStr">
         <is>
-          <t>2025-10-14 00:22:47</t>
+          <t>2025-10-16 03:37:04</t>
         </is>
       </c>
       <c r="AF6" s="11" t="n">
@@ -1091,12 +1091,12 @@
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>466100</t>
+          <t>125490</t>
         </is>
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>클로봇</t>
+          <t>한라캐스트</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
@@ -1111,45 +1111,45 @@
       </c>
       <c r="E7" s="6" t="inlineStr">
         <is>
-          <t>1차 매수선까지 68.8%</t>
+          <t>1차 매수선까지 72.8%</t>
         </is>
       </c>
       <c r="F7" s="7" t="n">
-        <v>39350</v>
+        <v>10940</v>
       </c>
       <c r="G7" s="7" t="n">
-        <v>35700</v>
+        <v>8690</v>
       </c>
       <c r="H7" s="7" t="n">
-        <v>41350</v>
+        <v>10940</v>
       </c>
       <c r="I7" s="7" t="n">
-        <v>29077.5</v>
+        <v>7903</v>
       </c>
       <c r="J7" s="7" t="n">
-        <v>23262</v>
+        <v>6322.400000000001</v>
       </c>
       <c r="K7" s="7" t="n">
-        <v>23312</v>
+        <v>6332.400000000001</v>
       </c>
       <c r="L7" s="8" t="n">
-        <v>0.6879718599862731</v>
+        <v>0.7276230181289872</v>
       </c>
       <c r="M7" s="9" t="inlineStr"/>
       <c r="N7" s="9" t="inlineStr"/>
       <c r="O7" s="7" t="n">
-        <v>20980.8</v>
+        <v>5699.160000000001</v>
       </c>
       <c r="P7" s="8" t="n">
-        <v>0.8755242888736369</v>
+        <v>0.9195811312544302</v>
       </c>
       <c r="Q7" s="9" t="inlineStr"/>
       <c r="R7" s="9" t="inlineStr"/>
       <c r="S7" s="7" t="n">
-        <v>18882.72</v>
+        <v>5129.244000000001</v>
       </c>
       <c r="T7" s="8" t="n">
-        <v>1.083915876526263</v>
+        <v>1.132867923616034</v>
       </c>
       <c r="U7" s="9" t="inlineStr"/>
       <c r="V7" s="9" t="inlineStr"/>
@@ -1163,11 +1163,11 @@
       <c r="AD7" s="9" t="inlineStr"/>
       <c r="AE7" s="10" t="inlineStr">
         <is>
-          <t>2025-10-14 00:22:47</t>
+          <t>2025-10-16 03:37:04</t>
         </is>
       </c>
       <c r="AF7" s="11" t="n">
-        <v>45943</v>
+        <v>45916</v>
       </c>
       <c r="AG7" s="6" t="inlineStr"/>
       <c r="AH7" s="6" t="inlineStr"/>
@@ -1175,12 +1175,12 @@
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>108490</t>
+          <t>466100</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>로보티즈</t>
+          <t>클로봇</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
@@ -1195,45 +1195,45 @@
       </c>
       <c r="E8" s="6" t="inlineStr">
         <is>
-          <t>1차 매수선까지 78.7%</t>
+          <t>1차 매수선까지 75.4%</t>
         </is>
       </c>
       <c r="F8" s="7" t="n">
-        <v>192100</v>
+        <v>43200</v>
       </c>
       <c r="G8" s="7" t="n">
-        <v>184000</v>
+        <v>40800</v>
       </c>
       <c r="H8" s="7" t="n">
-        <v>198700</v>
+        <v>44350</v>
       </c>
       <c r="I8" s="7" t="n">
-        <v>133759.7</v>
+        <v>30720</v>
       </c>
       <c r="J8" s="7" t="n">
-        <v>107007.76</v>
+        <v>24576</v>
       </c>
       <c r="K8" s="7" t="n">
-        <v>107507.76</v>
+        <v>24626</v>
       </c>
       <c r="L8" s="8" t="n">
-        <v>0.7868477587106268</v>
+        <v>0.7542434824981725</v>
       </c>
       <c r="M8" s="9" t="inlineStr"/>
       <c r="N8" s="9" t="inlineStr"/>
       <c r="O8" s="7" t="n">
-        <v>96756.98400000001</v>
+        <v>22163.4</v>
       </c>
       <c r="P8" s="8" t="n">
-        <v>0.9853863985673631</v>
+        <v>0.9491594249979695</v>
       </c>
       <c r="Q8" s="9" t="inlineStr"/>
       <c r="R8" s="9" t="inlineStr"/>
       <c r="S8" s="7" t="n">
-        <v>87081.28560000002</v>
+        <v>19947.06</v>
       </c>
       <c r="T8" s="8" t="n">
-        <v>1.20598488729707</v>
+        <v>1.165732694442188</v>
       </c>
       <c r="U8" s="9" t="inlineStr"/>
       <c r="V8" s="9" t="inlineStr"/>
@@ -1247,11 +1247,11 @@
       <c r="AD8" s="9" t="inlineStr"/>
       <c r="AE8" s="10" t="inlineStr">
         <is>
-          <t>2025-10-14 00:22:47</t>
+          <t>2025-10-16 03:37:04</t>
         </is>
       </c>
       <c r="AF8" s="11" t="n">
-        <v>45942</v>
+        <v>45943</v>
       </c>
       <c r="AG8" s="6" t="inlineStr"/>
       <c r="AH8" s="6" t="inlineStr"/>
@@ -1259,12 +1259,12 @@
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>005935</t>
+          <t>108490</t>
         </is>
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>삼성전자우</t>
+          <t>로보티즈</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
@@ -1279,45 +1279,45 @@
       </c>
       <c r="E9" s="6" t="inlineStr">
         <is>
-          <t>1차 매수선까지 39.9%</t>
+          <t>1차 매수선까지 75.3%</t>
         </is>
       </c>
       <c r="F9" s="7" t="n">
-        <v>73300</v>
+        <v>202500</v>
       </c>
       <c r="G9" s="7" t="n">
-        <v>71200</v>
+        <v>189600</v>
       </c>
       <c r="H9" s="7" t="n">
-        <v>73400</v>
+        <v>210000</v>
       </c>
       <c r="I9" s="7" t="n">
-        <v>65370</v>
+        <v>143733.05</v>
       </c>
       <c r="J9" s="7" t="n">
-        <v>52296</v>
+        <v>114986.44</v>
       </c>
       <c r="K9" s="7" t="n">
-        <v>52396</v>
+        <v>115486.44</v>
       </c>
       <c r="L9" s="8" t="n">
-        <v>0.3989617528055577</v>
+        <v>0.753452613137958</v>
       </c>
       <c r="M9" s="9" t="inlineStr"/>
       <c r="N9" s="9" t="inlineStr"/>
       <c r="O9" s="7" t="n">
-        <v>47156.4</v>
+        <v>103937.796</v>
       </c>
       <c r="P9" s="8" t="n">
-        <v>0.5544019475617306</v>
+        <v>0.9482806812643978</v>
       </c>
       <c r="Q9" s="9" t="inlineStr"/>
       <c r="R9" s="9" t="inlineStr"/>
       <c r="S9" s="7" t="n">
-        <v>42440.76</v>
+        <v>93544.01640000001</v>
       </c>
       <c r="T9" s="8" t="n">
-        <v>0.7271132750685897</v>
+        <v>1.164756312515997</v>
       </c>
       <c r="U9" s="9" t="inlineStr"/>
       <c r="V9" s="9" t="inlineStr"/>
@@ -1331,7 +1331,7 @@
       <c r="AD9" s="9" t="inlineStr"/>
       <c r="AE9" s="10" t="inlineStr">
         <is>
-          <t>2025-10-14 00:22:48</t>
+          <t>2025-10-16 03:37:05</t>
         </is>
       </c>
       <c r="AF9" s="11" t="n">
@@ -1343,12 +1343,12 @@
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>249420</t>
+          <t>005935</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>일동제약</t>
+          <t>삼성전자우</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
@@ -1363,45 +1363,45 @@
       </c>
       <c r="E10" s="6" t="inlineStr">
         <is>
-          <t>1차 매수선까지 15.5%</t>
+          <t>1차 매수선까지 38.0%</t>
         </is>
       </c>
       <c r="F10" s="7" t="n">
-        <v>24600</v>
+        <v>73900</v>
       </c>
       <c r="G10" s="7" t="n">
-        <v>24300</v>
+        <v>72400</v>
       </c>
       <c r="H10" s="7" t="n">
-        <v>26550</v>
+        <v>74000</v>
       </c>
       <c r="I10" s="7" t="n">
-        <v>26570</v>
+        <v>66800</v>
       </c>
       <c r="J10" s="7" t="n">
-        <v>21256</v>
+        <v>53440</v>
       </c>
       <c r="K10" s="7" t="n">
-        <v>21306</v>
+        <v>53540</v>
       </c>
       <c r="L10" s="8" t="n">
-        <v>0.1546043368065334</v>
+        <v>0.3802764288382518</v>
       </c>
       <c r="M10" s="9" t="inlineStr"/>
       <c r="N10" s="9" t="inlineStr"/>
       <c r="O10" s="7" t="n">
-        <v>19175.4</v>
+        <v>48186</v>
       </c>
       <c r="P10" s="8" t="n">
-        <v>0.2828937075628147</v>
+        <v>0.5336404764869463</v>
       </c>
       <c r="Q10" s="9" t="inlineStr"/>
       <c r="R10" s="9" t="inlineStr"/>
       <c r="S10" s="7" t="n">
-        <v>17257.86</v>
+        <v>43367.4</v>
       </c>
       <c r="T10" s="8" t="n">
-        <v>0.425437452847572</v>
+        <v>0.7040449738743848</v>
       </c>
       <c r="U10" s="9" t="inlineStr"/>
       <c r="V10" s="9" t="inlineStr"/>
@@ -1415,11 +1415,11 @@
       <c r="AD10" s="9" t="inlineStr"/>
       <c r="AE10" s="10" t="inlineStr">
         <is>
-          <t>2025-10-14 00:22:48</t>
+          <t>2025-10-16 03:37:05</t>
         </is>
       </c>
       <c r="AF10" s="11" t="n">
-        <v>45929</v>
+        <v>45942</v>
       </c>
       <c r="AG10" s="6" t="inlineStr"/>
       <c r="AH10" s="6" t="inlineStr"/>
@@ -1427,12 +1427,12 @@
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>041190</t>
+          <t>249420</t>
         </is>
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>우리기술투자</t>
+          <t>일동제약</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
@@ -1447,45 +1447,45 @@
       </c>
       <c r="E11" s="6" t="inlineStr">
         <is>
-          <t>1차 매수선까지 18.9%</t>
+          <t>1차 매수선까지 10.8%</t>
         </is>
       </c>
       <c r="F11" s="7" t="n">
-        <v>10420</v>
+        <v>23700</v>
       </c>
       <c r="G11" s="7" t="n">
-        <v>10270</v>
+        <v>23600</v>
       </c>
       <c r="H11" s="7" t="n">
-        <v>10780</v>
+        <v>24400</v>
       </c>
       <c r="I11" s="7" t="n">
-        <v>10939.5</v>
+        <v>26675</v>
       </c>
       <c r="J11" s="7" t="n">
-        <v>8751.6</v>
+        <v>21340</v>
       </c>
       <c r="K11" s="7" t="n">
-        <v>8761.6</v>
+        <v>21390</v>
       </c>
       <c r="L11" s="8" t="n">
-        <v>0.1892804967129291</v>
+        <v>0.1079943899018233</v>
       </c>
       <c r="M11" s="9" t="inlineStr"/>
       <c r="N11" s="9" t="inlineStr"/>
       <c r="O11" s="7" t="n">
-        <v>7885.440000000001</v>
+        <v>19251</v>
       </c>
       <c r="P11" s="8" t="n">
-        <v>0.3214227741254768</v>
+        <v>0.2311048776686925</v>
       </c>
       <c r="Q11" s="9" t="inlineStr"/>
       <c r="R11" s="9" t="inlineStr"/>
       <c r="S11" s="7" t="n">
-        <v>7096.896000000001</v>
+        <v>17325.9</v>
       </c>
       <c r="T11" s="8" t="n">
-        <v>0.4682475268060852</v>
+        <v>0.3678943085207694</v>
       </c>
       <c r="U11" s="9" t="inlineStr"/>
       <c r="V11" s="9" t="inlineStr"/>
@@ -1499,7 +1499,7 @@
       <c r="AD11" s="9" t="inlineStr"/>
       <c r="AE11" s="10" t="inlineStr">
         <is>
-          <t>2025-10-14 00:22:48</t>
+          <t>2025-10-16 03:37:05</t>
         </is>
       </c>
       <c r="AF11" s="11" t="n">
@@ -1511,12 +1511,12 @@
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>060250</t>
+          <t>041190</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>NHN KCP</t>
+          <t>우리기술투자</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
@@ -1531,45 +1531,45 @@
       </c>
       <c r="E12" s="6" t="inlineStr">
         <is>
-          <t>1차 매수선까지 39.3%</t>
+          <t>1차 매수선까지 15.7%</t>
         </is>
       </c>
       <c r="F12" s="7" t="n">
-        <v>17850</v>
+        <v>10120</v>
       </c>
       <c r="G12" s="7" t="n">
-        <v>17610</v>
+        <v>9920</v>
       </c>
       <c r="H12" s="7" t="n">
-        <v>18270</v>
+        <v>10180</v>
       </c>
       <c r="I12" s="7" t="n">
-        <v>15949.5</v>
+        <v>10922.5</v>
       </c>
       <c r="J12" s="7" t="n">
-        <v>12759.6</v>
+        <v>8738</v>
       </c>
       <c r="K12" s="7" t="n">
-        <v>12809.6</v>
+        <v>8748</v>
       </c>
       <c r="L12" s="8" t="n">
-        <v>0.3934861353984511</v>
+        <v>0.1568358481938729</v>
       </c>
       <c r="M12" s="9" t="inlineStr"/>
       <c r="N12" s="9" t="inlineStr"/>
       <c r="O12" s="7" t="n">
-        <v>11528.64</v>
+        <v>7873.2</v>
       </c>
       <c r="P12" s="8" t="n">
-        <v>0.548317928220501</v>
+        <v>0.2853731646598588</v>
       </c>
       <c r="Q12" s="9" t="inlineStr"/>
       <c r="R12" s="9" t="inlineStr"/>
       <c r="S12" s="7" t="n">
-        <v>10375.776</v>
+        <v>7085.88</v>
       </c>
       <c r="T12" s="8" t="n">
-        <v>0.7203532535783345</v>
+        <v>0.4281924051776208</v>
       </c>
       <c r="U12" s="9" t="inlineStr"/>
       <c r="V12" s="9" t="inlineStr"/>
@@ -1583,11 +1583,11 @@
       <c r="AD12" s="9" t="inlineStr"/>
       <c r="AE12" s="10" t="inlineStr">
         <is>
-          <t>2025-10-14 00:22:49</t>
+          <t>2025-10-16 03:37:06</t>
         </is>
       </c>
       <c r="AF12" s="11" t="n">
-        <v>45926</v>
+        <v>45929</v>
       </c>
       <c r="AG12" s="6" t="inlineStr"/>
       <c r="AH12" s="6" t="inlineStr"/>
@@ -1595,12 +1595,12 @@
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>035720</t>
+          <t>060250</t>
         </is>
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>카카오</t>
+          <t>NHN KCP</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
@@ -1615,45 +1615,45 @@
       </c>
       <c r="E13" s="6" t="inlineStr">
         <is>
-          <t>1차 매수선까지 20.2%</t>
+          <t>1차 매수선까지 33.8%</t>
         </is>
       </c>
       <c r="F13" s="7" t="n">
-        <v>59800</v>
+        <v>17620</v>
       </c>
       <c r="G13" s="7" t="n">
-        <v>59600</v>
+        <v>16700</v>
       </c>
       <c r="H13" s="7" t="n">
-        <v>60700</v>
+        <v>18340</v>
       </c>
       <c r="I13" s="7" t="n">
-        <v>62120</v>
+        <v>16396.5</v>
       </c>
       <c r="J13" s="7" t="n">
-        <v>49696</v>
+        <v>13117.2</v>
       </c>
       <c r="K13" s="7" t="n">
-        <v>49746</v>
+        <v>13167.2</v>
       </c>
       <c r="L13" s="8" t="n">
-        <v>0.2021067020463957</v>
+        <v>0.3381736435992465</v>
       </c>
       <c r="M13" s="9" t="inlineStr"/>
       <c r="N13" s="9" t="inlineStr"/>
       <c r="O13" s="7" t="n">
-        <v>44771.4</v>
+        <v>11850.48</v>
       </c>
       <c r="P13" s="8" t="n">
-        <v>0.3356741133848841</v>
+        <v>0.4868596039991628</v>
       </c>
       <c r="Q13" s="9" t="inlineStr"/>
       <c r="R13" s="9" t="inlineStr"/>
       <c r="S13" s="7" t="n">
-        <v>40294.26</v>
+        <v>10665.432</v>
       </c>
       <c r="T13" s="8" t="n">
-        <v>0.4840823482054267</v>
+        <v>0.6520662266657365</v>
       </c>
       <c r="U13" s="9" t="inlineStr"/>
       <c r="V13" s="9" t="inlineStr"/>
@@ -1667,7 +1667,7 @@
       <c r="AD13" s="9" t="inlineStr"/>
       <c r="AE13" s="10" t="inlineStr">
         <is>
-          <t>2025-10-14 00:22:49</t>
+          <t>2025-10-16 03:37:06</t>
         </is>
       </c>
       <c r="AF13" s="11" t="n">
@@ -1679,12 +1679,12 @@
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>277810</t>
+          <t>035720</t>
         </is>
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>레인보우로보틱스</t>
+          <t>카카오</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
@@ -1699,45 +1699,45 @@
       </c>
       <c r="E14" s="6" t="inlineStr">
         <is>
-          <t>1차 매수선까지 40.9%</t>
+          <t>1차 매수선까지 19.7%</t>
         </is>
       </c>
       <c r="F14" s="7" t="n">
-        <v>344000</v>
+        <v>59600</v>
       </c>
       <c r="G14" s="7" t="n">
-        <v>316500</v>
+        <v>59100</v>
       </c>
       <c r="H14" s="7" t="n">
-        <v>354500</v>
+        <v>60200</v>
       </c>
       <c r="I14" s="7" t="n">
-        <v>304450</v>
+        <v>62195</v>
       </c>
       <c r="J14" s="7" t="n">
-        <v>243560</v>
+        <v>49756</v>
       </c>
       <c r="K14" s="7" t="n">
-        <v>244060</v>
+        <v>49806</v>
       </c>
       <c r="L14" s="8" t="n">
-        <v>0.4094894698025076</v>
+        <v>0.1966429747419989</v>
       </c>
       <c r="M14" s="9" t="inlineStr"/>
       <c r="N14" s="9" t="inlineStr"/>
       <c r="O14" s="7" t="n">
-        <v>219654</v>
+        <v>44825.4</v>
       </c>
       <c r="P14" s="8" t="n">
-        <v>0.5660994108916751</v>
+        <v>0.3296033052688877</v>
       </c>
       <c r="Q14" s="9" t="inlineStr"/>
       <c r="R14" s="9" t="inlineStr"/>
       <c r="S14" s="7" t="n">
-        <v>197688.6</v>
+        <v>40342.86</v>
       </c>
       <c r="T14" s="8" t="n">
-        <v>0.7401104565463057</v>
+        <v>0.4773370058543197</v>
       </c>
       <c r="U14" s="9" t="inlineStr"/>
       <c r="V14" s="9" t="inlineStr"/>
@@ -1751,11 +1751,11 @@
       <c r="AD14" s="9" t="inlineStr"/>
       <c r="AE14" s="10" t="inlineStr">
         <is>
-          <t>2025-10-14 00:22:49</t>
+          <t>2025-10-16 03:37:06</t>
         </is>
       </c>
       <c r="AF14" s="11" t="n">
-        <v>45925</v>
+        <v>45926</v>
       </c>
       <c r="AG14" s="6" t="inlineStr"/>
       <c r="AH14" s="6" t="inlineStr"/>
@@ -1763,12 +1763,12 @@
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
         <is>
-          <t>196170</t>
+          <t>277810</t>
         </is>
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>알테오젠</t>
+          <t>레인보우로보틱스</t>
         </is>
       </c>
       <c r="C15" s="5" t="inlineStr">
@@ -1783,45 +1783,45 @@
       </c>
       <c r="E15" s="6" t="inlineStr">
         <is>
-          <t>1차 매수선까지 17.4%</t>
+          <t>1차 매수선까지 41.4%</t>
         </is>
       </c>
       <c r="F15" s="7" t="n">
-        <v>444000</v>
+        <v>352000</v>
       </c>
       <c r="G15" s="7" t="n">
-        <v>442500</v>
+        <v>331000</v>
       </c>
       <c r="H15" s="7" t="n">
-        <v>455500</v>
+        <v>353500</v>
       </c>
       <c r="I15" s="7" t="n">
-        <v>472225</v>
+        <v>310575</v>
       </c>
       <c r="J15" s="7" t="n">
-        <v>377780</v>
+        <v>248460</v>
       </c>
       <c r="K15" s="7" t="n">
-        <v>378280</v>
+        <v>248960</v>
       </c>
       <c r="L15" s="8" t="n">
-        <v>0.1737337422015438</v>
+        <v>0.4138817480719794</v>
       </c>
       <c r="M15" s="9" t="inlineStr"/>
       <c r="N15" s="9" t="inlineStr"/>
       <c r="O15" s="7" t="n">
-        <v>340452</v>
+        <v>224064</v>
       </c>
       <c r="P15" s="8" t="n">
-        <v>0.3041486024461598</v>
+        <v>0.5709797200799771</v>
       </c>
       <c r="Q15" s="9" t="inlineStr"/>
       <c r="R15" s="9" t="inlineStr"/>
       <c r="S15" s="7" t="n">
-        <v>306406.8</v>
+        <v>201657.6</v>
       </c>
       <c r="T15" s="8" t="n">
-        <v>0.4490540027179554</v>
+        <v>0.7455330223110856</v>
       </c>
       <c r="U15" s="9" t="inlineStr"/>
       <c r="V15" s="9" t="inlineStr"/>
@@ -1835,11 +1835,11 @@
       <c r="AD15" s="9" t="inlineStr"/>
       <c r="AE15" s="10" t="inlineStr">
         <is>
-          <t>2025-10-14 00:22:50</t>
+          <t>2025-10-16 03:37:07</t>
         </is>
       </c>
       <c r="AF15" s="11" t="n">
-        <v>45924</v>
+        <v>45925</v>
       </c>
       <c r="AG15" s="6" t="inlineStr"/>
       <c r="AH15" s="6" t="inlineStr"/>
@@ -1847,12 +1847,12 @@
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>068270</t>
+          <t>196170</t>
         </is>
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>셀트리온</t>
+          <t>알테오젠</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
@@ -1867,45 +1867,45 @@
       </c>
       <c r="E16" s="6" t="inlineStr">
         <is>
-          <t>1차 매수선까지 23.0%</t>
+          <t>1차 매수선까지 19.0%</t>
         </is>
       </c>
       <c r="F16" s="7" t="n">
-        <v>170900</v>
+        <v>447500</v>
       </c>
       <c r="G16" s="7" t="n">
-        <v>170000</v>
+        <v>443500</v>
       </c>
       <c r="H16" s="7" t="n">
-        <v>172000</v>
+        <v>452500</v>
       </c>
       <c r="I16" s="7" t="n">
-        <v>173120</v>
+        <v>469300</v>
       </c>
       <c r="J16" s="7" t="n">
-        <v>138496</v>
+        <v>375440</v>
       </c>
       <c r="K16" s="7" t="n">
-        <v>138996</v>
+        <v>375940</v>
       </c>
       <c r="L16" s="8" t="n">
-        <v>0.2295317850873407</v>
+        <v>0.1903495238601905</v>
       </c>
       <c r="M16" s="9" t="inlineStr"/>
       <c r="N16" s="9" t="inlineStr"/>
       <c r="O16" s="7" t="n">
-        <v>125096.4</v>
+        <v>338346</v>
       </c>
       <c r="P16" s="8" t="n">
-        <v>0.3661464278748228</v>
+        <v>0.3226105820668783</v>
       </c>
       <c r="Q16" s="9" t="inlineStr"/>
       <c r="R16" s="9" t="inlineStr"/>
       <c r="S16" s="7" t="n">
-        <v>112586.76</v>
+        <v>304511.4</v>
       </c>
       <c r="T16" s="8" t="n">
-        <v>0.5179404754164698</v>
+        <v>0.4695673134076424</v>
       </c>
       <c r="U16" s="9" t="inlineStr"/>
       <c r="V16" s="9" t="inlineStr"/>
@@ -1919,11 +1919,11 @@
       <c r="AD16" s="9" t="inlineStr"/>
       <c r="AE16" s="10" t="inlineStr">
         <is>
-          <t>2025-10-14 00:22:50</t>
+          <t>2025-10-16 03:37:07</t>
         </is>
       </c>
       <c r="AF16" s="11" t="n">
-        <v>45923</v>
+        <v>45924</v>
       </c>
       <c r="AG16" s="6" t="inlineStr"/>
       <c r="AH16" s="6" t="inlineStr"/>
@@ -1931,12 +1931,12 @@
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
         <is>
-          <t>347850</t>
+          <t>068270</t>
         </is>
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>디앤디파마텍</t>
+          <t>셀트리온</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr">
@@ -1951,45 +1951,45 @@
       </c>
       <c r="E17" s="6" t="inlineStr">
         <is>
-          <t>1차 매수선까지 26.8%</t>
+          <t>1차 매수선까지 23.3%</t>
         </is>
       </c>
       <c r="F17" s="7" t="n">
-        <v>186400</v>
+        <v>171400</v>
       </c>
       <c r="G17" s="7" t="n">
-        <v>185500</v>
+        <v>169000</v>
       </c>
       <c r="H17" s="7" t="n">
-        <v>195900</v>
+        <v>172500</v>
       </c>
       <c r="I17" s="7" t="n">
-        <v>183140</v>
+        <v>173080</v>
       </c>
       <c r="J17" s="7" t="n">
-        <v>146512</v>
+        <v>138464</v>
       </c>
       <c r="K17" s="7" t="n">
-        <v>147012</v>
+        <v>138964</v>
       </c>
       <c r="L17" s="8" t="n">
-        <v>0.2679237069082796</v>
+        <v>0.2334129702656803</v>
       </c>
       <c r="M17" s="9" t="inlineStr"/>
       <c r="N17" s="9" t="inlineStr"/>
       <c r="O17" s="7" t="n">
-        <v>132310.8</v>
+        <v>125067.6</v>
       </c>
       <c r="P17" s="8" t="n">
-        <v>0.4088041187869771</v>
+        <v>0.3704588558507558</v>
       </c>
       <c r="Q17" s="9" t="inlineStr"/>
       <c r="R17" s="9" t="inlineStr"/>
       <c r="S17" s="7" t="n">
-        <v>119079.72</v>
+        <v>112560.84</v>
       </c>
       <c r="T17" s="8" t="n">
-        <v>0.5653379097633079</v>
+        <v>0.5227320620563953</v>
       </c>
       <c r="U17" s="9" t="inlineStr"/>
       <c r="V17" s="9" t="inlineStr"/>
@@ -2003,7 +2003,7 @@
       <c r="AD17" s="9" t="inlineStr"/>
       <c r="AE17" s="10" t="inlineStr">
         <is>
-          <t>2025-10-14 00:22:50</t>
+          <t>2025-10-16 03:37:07</t>
         </is>
       </c>
       <c r="AF17" s="11" t="n">
@@ -2015,12 +2015,12 @@
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>000250</t>
+          <t>347850</t>
         </is>
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>삼천당제약</t>
+          <t>디앤디파마텍</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
@@ -2035,45 +2035,45 @@
       </c>
       <c r="E18" s="6" t="inlineStr">
         <is>
-          <t>1차 매수선까지 15.1%</t>
+          <t>1차 매수선까지 16.6%</t>
         </is>
       </c>
       <c r="F18" s="7" t="n">
-        <v>203000</v>
+        <v>172400</v>
       </c>
       <c r="G18" s="7" t="n">
-        <v>201000</v>
+        <v>172300</v>
       </c>
       <c r="H18" s="7" t="n">
-        <v>207500</v>
+        <v>181500</v>
       </c>
       <c r="I18" s="7" t="n">
-        <v>219750</v>
+        <v>184230</v>
       </c>
       <c r="J18" s="7" t="n">
-        <v>175800</v>
+        <v>147384</v>
       </c>
       <c r="K18" s="7" t="n">
-        <v>176300</v>
+        <v>147884</v>
       </c>
       <c r="L18" s="8" t="n">
-        <v>0.1514463981849121</v>
+        <v>0.1657785832138703</v>
       </c>
       <c r="M18" s="9" t="inlineStr"/>
       <c r="N18" s="9" t="inlineStr"/>
       <c r="O18" s="7" t="n">
-        <v>158670</v>
+        <v>133095.6</v>
       </c>
       <c r="P18" s="8" t="n">
-        <v>0.2793848868721246</v>
+        <v>0.2953095369043003</v>
       </c>
       <c r="Q18" s="9" t="inlineStr"/>
       <c r="R18" s="9" t="inlineStr"/>
       <c r="S18" s="7" t="n">
-        <v>142803</v>
+        <v>119786.04</v>
       </c>
       <c r="T18" s="8" t="n">
-        <v>0.4215387631912495</v>
+        <v>0.4392328187825559</v>
       </c>
       <c r="U18" s="9" t="inlineStr"/>
       <c r="V18" s="9" t="inlineStr"/>
@@ -2087,11 +2087,11 @@
       <c r="AD18" s="9" t="inlineStr"/>
       <c r="AE18" s="10" t="inlineStr">
         <is>
-          <t>2025-10-14 00:22:51</t>
+          <t>2025-10-16 03:37:08</t>
         </is>
       </c>
       <c r="AF18" s="11" t="n">
-        <v>45919</v>
+        <v>45923</v>
       </c>
       <c r="AG18" s="6" t="inlineStr"/>
       <c r="AH18" s="6" t="inlineStr"/>
@@ -2099,12 +2099,12 @@
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
         <is>
-          <t>064260</t>
+          <t>000250</t>
         </is>
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>다날</t>
+          <t>삼천당제약</t>
         </is>
       </c>
       <c r="C19" s="5" t="inlineStr">
@@ -2119,45 +2119,45 @@
       </c>
       <c r="E19" s="6" t="inlineStr">
         <is>
-          <t>1차 매수선까지 19.0%</t>
+          <t>1차 매수선까지 14.3%</t>
         </is>
       </c>
       <c r="F19" s="7" t="n">
-        <v>9230</v>
+        <v>201500</v>
       </c>
       <c r="G19" s="7" t="n">
-        <v>9230</v>
+        <v>197700</v>
       </c>
       <c r="H19" s="7" t="n">
-        <v>10020</v>
+        <v>204000</v>
       </c>
       <c r="I19" s="7" t="n">
-        <v>9681</v>
+        <v>219750</v>
       </c>
       <c r="J19" s="7" t="n">
-        <v>7744.8</v>
+        <v>175800</v>
       </c>
       <c r="K19" s="7" t="n">
-        <v>7754.8</v>
+        <v>176300</v>
       </c>
       <c r="L19" s="8" t="n">
-        <v>0.1902305668747098</v>
+        <v>0.1429381735677822</v>
       </c>
       <c r="M19" s="9" t="inlineStr"/>
       <c r="N19" s="9" t="inlineStr"/>
       <c r="O19" s="7" t="n">
-        <v>6979.320000000001</v>
+        <v>158670</v>
       </c>
       <c r="P19" s="8" t="n">
-        <v>0.3224784076385664</v>
+        <v>0.2699313039642024</v>
       </c>
       <c r="Q19" s="9" t="inlineStr"/>
       <c r="R19" s="9" t="inlineStr"/>
       <c r="S19" s="7" t="n">
-        <v>6281.388000000001</v>
+        <v>142803</v>
       </c>
       <c r="T19" s="8" t="n">
-        <v>0.4694204529317404</v>
+        <v>0.4110347821824472</v>
       </c>
       <c r="U19" s="9" t="inlineStr"/>
       <c r="V19" s="9" t="inlineStr"/>
@@ -2171,7 +2171,7 @@
       <c r="AD19" s="9" t="inlineStr"/>
       <c r="AE19" s="10" t="inlineStr">
         <is>
-          <t>2025-10-14 00:22:51</t>
+          <t>2025-10-16 03:37:08</t>
         </is>
       </c>
       <c r="AF19" s="11" t="n">
@@ -2183,12 +2183,12 @@
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
         <is>
-          <t>064350</t>
+          <t>064260</t>
         </is>
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>현대로템</t>
+          <t>다날</t>
         </is>
       </c>
       <c r="C20" s="5" t="inlineStr">
@@ -2203,45 +2203,45 @@
       </c>
       <c r="E20" s="6" t="inlineStr">
         <is>
-          <t>1차 매수선까지 20.3%</t>
+          <t>1차 매수선까지 24.3%</t>
         </is>
       </c>
       <c r="F20" s="7" t="n">
-        <v>210000</v>
+        <v>9720</v>
       </c>
       <c r="G20" s="7" t="n">
-        <v>208500</v>
+        <v>9630</v>
       </c>
       <c r="H20" s="7" t="n">
-        <v>220000</v>
+        <v>10330</v>
       </c>
       <c r="I20" s="7" t="n">
-        <v>217525</v>
+        <v>9765.5</v>
       </c>
       <c r="J20" s="7" t="n">
-        <v>174020</v>
+        <v>7812.400000000001</v>
       </c>
       <c r="K20" s="7" t="n">
-        <v>174520</v>
+        <v>7822.400000000001</v>
       </c>
       <c r="L20" s="8" t="n">
-        <v>0.2033004813201925</v>
+        <v>0.2425853957864593</v>
       </c>
       <c r="M20" s="9" t="inlineStr"/>
       <c r="N20" s="9" t="inlineStr"/>
       <c r="O20" s="7" t="n">
-        <v>157068</v>
+        <v>7040.160000000001</v>
       </c>
       <c r="P20" s="8" t="n">
-        <v>0.3370005348002139</v>
+        <v>0.3806504397627325</v>
       </c>
       <c r="Q20" s="9" t="inlineStr"/>
       <c r="R20" s="9" t="inlineStr"/>
       <c r="S20" s="7" t="n">
-        <v>141361.2</v>
+        <v>6336.144000000001</v>
       </c>
       <c r="T20" s="8" t="n">
-        <v>0.4855561497780154</v>
+        <v>0.5340560441808136</v>
       </c>
       <c r="U20" s="9" t="inlineStr"/>
       <c r="V20" s="9" t="inlineStr"/>
@@ -2255,7 +2255,7 @@
       <c r="AD20" s="9" t="inlineStr"/>
       <c r="AE20" s="10" t="inlineStr">
         <is>
-          <t>2025-10-14 00:22:51</t>
+          <t>2025-10-16 03:37:08</t>
         </is>
       </c>
       <c r="AF20" s="11" t="n">
@@ -2267,12 +2267,12 @@
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
         <is>
-          <t>090360</t>
+          <t>064350</t>
         </is>
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>로보스타</t>
+          <t>현대로템</t>
         </is>
       </c>
       <c r="C21" s="5" t="inlineStr">
@@ -2287,45 +2287,45 @@
       </c>
       <c r="E21" s="6" t="inlineStr">
         <is>
-          <t>1차 매수선까지 44.7%</t>
+          <t>1차 매수선까지 21.9%</t>
         </is>
       </c>
       <c r="F21" s="7" t="n">
-        <v>48450</v>
+        <v>213000</v>
       </c>
       <c r="G21" s="7" t="n">
-        <v>45650</v>
+        <v>202000</v>
       </c>
       <c r="H21" s="7" t="n">
-        <v>49900</v>
+        <v>214500</v>
       </c>
       <c r="I21" s="7" t="n">
-        <v>41790</v>
+        <v>217750</v>
       </c>
       <c r="J21" s="7" t="n">
-        <v>33432</v>
+        <v>174200</v>
       </c>
       <c r="K21" s="7" t="n">
-        <v>33482</v>
+        <v>174700</v>
       </c>
       <c r="L21" s="8" t="n">
-        <v>0.447046174063676</v>
+        <v>0.2192329708070979</v>
       </c>
       <c r="M21" s="9" t="inlineStr"/>
       <c r="N21" s="9" t="inlineStr"/>
       <c r="O21" s="7" t="n">
-        <v>30133.8</v>
+        <v>157230</v>
       </c>
       <c r="P21" s="8" t="n">
-        <v>0.6078290822929734</v>
+        <v>0.3547033008967755</v>
       </c>
       <c r="Q21" s="9" t="inlineStr"/>
       <c r="R21" s="9" t="inlineStr"/>
       <c r="S21" s="7" t="n">
-        <v>27120.42</v>
+        <v>141507</v>
       </c>
       <c r="T21" s="8" t="n">
-        <v>0.7864767581033039</v>
+        <v>0.505225889885306</v>
       </c>
       <c r="U21" s="9" t="inlineStr"/>
       <c r="V21" s="9" t="inlineStr"/>
@@ -2339,7 +2339,7 @@
       <c r="AD21" s="9" t="inlineStr"/>
       <c r="AE21" s="10" t="inlineStr">
         <is>
-          <t>2025-10-14 00:22:52</t>
+          <t>2025-10-16 03:37:09</t>
         </is>
       </c>
       <c r="AF21" s="11" t="n">
@@ -2351,12 +2351,12 @@
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>047810</t>
+          <t>090360</t>
         </is>
       </c>
       <c r="B22" s="5" t="inlineStr">
         <is>
-          <t>한국항공우주</t>
+          <t>로보스타</t>
         </is>
       </c>
       <c r="C22" s="5" t="inlineStr">
@@ -2371,45 +2371,45 @@
       </c>
       <c r="E22" s="6" t="inlineStr">
         <is>
-          <t>1차 매수선까지 20.7%</t>
+          <t>1차 매수선까지 80.9%</t>
         </is>
       </c>
       <c r="F22" s="7" t="n">
-        <v>101400</v>
+        <v>65700</v>
       </c>
       <c r="G22" s="7" t="n">
-        <v>100600</v>
+        <v>61400</v>
       </c>
       <c r="H22" s="7" t="n">
-        <v>106500</v>
+        <v>68300</v>
       </c>
       <c r="I22" s="7" t="n">
-        <v>104925</v>
+        <v>45325</v>
       </c>
       <c r="J22" s="7" t="n">
-        <v>83940</v>
+        <v>36260</v>
       </c>
       <c r="K22" s="7" t="n">
-        <v>84040</v>
+        <v>36310</v>
       </c>
       <c r="L22" s="8" t="n">
-        <v>0.2065683008091385</v>
+        <v>0.8094188928669788</v>
       </c>
       <c r="M22" s="9" t="inlineStr"/>
       <c r="N22" s="9" t="inlineStr"/>
       <c r="O22" s="7" t="n">
-        <v>75636</v>
+        <v>32679</v>
       </c>
       <c r="P22" s="8" t="n">
-        <v>0.3406314453434872</v>
+        <v>1.010465436518865</v>
       </c>
       <c r="Q22" s="9" t="inlineStr"/>
       <c r="R22" s="9" t="inlineStr"/>
       <c r="S22" s="7" t="n">
-        <v>68072.40000000001</v>
+        <v>29411.1</v>
       </c>
       <c r="T22" s="8" t="n">
-        <v>0.4895904948260967</v>
+        <v>1.233850485020961</v>
       </c>
       <c r="U22" s="9" t="inlineStr"/>
       <c r="V22" s="9" t="inlineStr"/>
@@ -2423,7 +2423,7 @@
       <c r="AD22" s="9" t="inlineStr"/>
       <c r="AE22" s="10" t="inlineStr">
         <is>
-          <t>2025-10-14 00:22:52</t>
+          <t>2025-10-16 03:37:09</t>
         </is>
       </c>
       <c r="AF22" s="11" t="n">
@@ -2435,12 +2435,12 @@
     <row r="23">
       <c r="A23" s="5" t="inlineStr">
         <is>
-          <t>042660</t>
+          <t>047810</t>
         </is>
       </c>
       <c r="B23" s="5" t="inlineStr">
         <is>
-          <t>한화오션</t>
+          <t>한국항공우주</t>
         </is>
       </c>
       <c r="C23" s="5" t="inlineStr">
@@ -2455,45 +2455,45 @@
       </c>
       <c r="E23" s="6" t="inlineStr">
         <is>
-          <t>1차 매수선까지 23.7%</t>
+          <t>1차 매수선까지 19.2%</t>
         </is>
       </c>
       <c r="F23" s="7" t="n">
-        <v>109400</v>
+        <v>100500</v>
       </c>
       <c r="G23" s="7" t="n">
-        <v>107700</v>
+        <v>98600</v>
       </c>
       <c r="H23" s="7" t="n">
-        <v>113000</v>
+        <v>101300</v>
       </c>
       <c r="I23" s="7" t="n">
-        <v>110385</v>
+        <v>105260</v>
       </c>
       <c r="J23" s="7" t="n">
-        <v>88308</v>
+        <v>84208</v>
       </c>
       <c r="K23" s="7" t="n">
-        <v>88408</v>
+        <v>84308</v>
       </c>
       <c r="L23" s="8" t="n">
-        <v>0.23744457515157</v>
+        <v>0.1920576932200978</v>
       </c>
       <c r="M23" s="9" t="inlineStr"/>
       <c r="N23" s="9" t="inlineStr"/>
       <c r="O23" s="7" t="n">
-        <v>79567.2</v>
+        <v>75877.2</v>
       </c>
       <c r="P23" s="8" t="n">
-        <v>0.3749384168350778</v>
+        <v>0.3245085480223309</v>
       </c>
       <c r="Q23" s="9" t="inlineStr"/>
       <c r="R23" s="9" t="inlineStr"/>
       <c r="S23" s="7" t="n">
-        <v>71610.48</v>
+        <v>68289.48</v>
       </c>
       <c r="T23" s="8" t="n">
-        <v>0.5277093520389754</v>
+        <v>0.4716761644692566</v>
       </c>
       <c r="U23" s="9" t="inlineStr"/>
       <c r="V23" s="9" t="inlineStr"/>
@@ -2507,11 +2507,11 @@
       <c r="AD23" s="9" t="inlineStr"/>
       <c r="AE23" s="10" t="inlineStr">
         <is>
-          <t>2025-10-14 00:22:52</t>
+          <t>2025-10-16 03:37:10</t>
         </is>
       </c>
       <c r="AF23" s="11" t="n">
-        <v>45917</v>
+        <v>45919</v>
       </c>
       <c r="AG23" s="6" t="inlineStr"/>
       <c r="AH23" s="6" t="inlineStr"/>
@@ -2519,12 +2519,12 @@
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>125490</t>
+          <t>042660</t>
         </is>
       </c>
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>한라캐스트</t>
+          <t>한화오션</t>
         </is>
       </c>
       <c r="C24" s="5" t="inlineStr">
@@ -2539,45 +2539,45 @@
       </c>
       <c r="E24" s="6" t="inlineStr">
         <is>
-          <t>1차 매수선까지 46.6%</t>
+          <t>1차 매수선까지 20.4%</t>
         </is>
       </c>
       <c r="F24" s="7" t="n">
-        <v>8800</v>
+        <v>105800</v>
       </c>
       <c r="G24" s="7" t="n">
-        <v>8140</v>
+        <v>102200</v>
       </c>
       <c r="H24" s="7" t="n">
-        <v>8910</v>
+        <v>106800</v>
       </c>
       <c r="I24" s="7" t="n">
-        <v>7491</v>
+        <v>109730</v>
       </c>
       <c r="J24" s="7" t="n">
-        <v>5992.8</v>
+        <v>87784</v>
       </c>
       <c r="K24" s="7" t="n">
-        <v>6002.8</v>
+        <v>87884</v>
       </c>
       <c r="L24" s="8" t="n">
-        <v>0.4659825414806424</v>
+        <v>0.2038596331527923</v>
       </c>
       <c r="M24" s="9" t="inlineStr"/>
       <c r="N24" s="9" t="inlineStr"/>
       <c r="O24" s="7" t="n">
-        <v>5402.52</v>
+        <v>79095.60000000001</v>
       </c>
       <c r="P24" s="8" t="n">
-        <v>0.6288694905340469</v>
+        <v>0.3376218146142136</v>
       </c>
       <c r="Q24" s="9" t="inlineStr"/>
       <c r="R24" s="9" t="inlineStr"/>
       <c r="S24" s="7" t="n">
-        <v>4862.268000000001</v>
+        <v>71186.04000000001</v>
       </c>
       <c r="T24" s="8" t="n">
-        <v>0.8098549894822742</v>
+        <v>0.4862464606824594</v>
       </c>
       <c r="U24" s="9" t="inlineStr"/>
       <c r="V24" s="9" t="inlineStr"/>
@@ -2591,11 +2591,11 @@
       <c r="AD24" s="9" t="inlineStr"/>
       <c r="AE24" s="10" t="inlineStr">
         <is>
-          <t>2025-10-14 00:22:53</t>
+          <t>2025-10-16 03:37:10</t>
         </is>
       </c>
       <c r="AF24" s="11" t="n">
-        <v>45916</v>
+        <v>45917</v>
       </c>
       <c r="AG24" s="6" t="inlineStr"/>
       <c r="AH24" s="6" t="inlineStr"/>
@@ -2623,45 +2623,45 @@
       </c>
       <c r="E25" s="6" t="inlineStr">
         <is>
-          <t>1차 매수선까지 17.4%</t>
+          <t>1차 매수선까지 16.3%</t>
         </is>
       </c>
       <c r="F25" s="7" t="n">
-        <v>189700</v>
+        <v>191500</v>
       </c>
       <c r="G25" s="7" t="n">
-        <v>187900</v>
+        <v>189100</v>
       </c>
       <c r="H25" s="7" t="n">
-        <v>199000</v>
+        <v>198700</v>
       </c>
       <c r="I25" s="7" t="n">
-        <v>201270</v>
+        <v>205270</v>
       </c>
       <c r="J25" s="7" t="n">
-        <v>161016</v>
+        <v>164216</v>
       </c>
       <c r="K25" s="7" t="n">
-        <v>161516</v>
+        <v>164716</v>
       </c>
       <c r="L25" s="8" t="n">
-        <v>0.174496644295302</v>
+        <v>0.1626071541319605</v>
       </c>
       <c r="M25" s="9" t="inlineStr"/>
       <c r="N25" s="9" t="inlineStr"/>
       <c r="O25" s="7" t="n">
-        <v>145364.4</v>
+        <v>148244.4</v>
       </c>
       <c r="P25" s="8" t="n">
-        <v>0.3049962714392245</v>
+        <v>0.2917857268132894</v>
       </c>
       <c r="Q25" s="9" t="inlineStr"/>
       <c r="R25" s="9" t="inlineStr"/>
       <c r="S25" s="7" t="n">
-        <v>130827.96</v>
+        <v>133419.96</v>
       </c>
       <c r="T25" s="8" t="n">
-        <v>0.4499958571546939</v>
+        <v>0.4353174742369883</v>
       </c>
       <c r="U25" s="9" t="inlineStr"/>
       <c r="V25" s="9" t="inlineStr"/>
@@ -2675,7 +2675,7 @@
       <c r="AD25" s="9" t="inlineStr"/>
       <c r="AE25" s="10" t="inlineStr">
         <is>
-          <t>2025-10-14 00:22:53</t>
+          <t>2025-10-16 03:37:10</t>
         </is>
       </c>
       <c r="AF25" s="11" t="n">
@@ -2707,45 +2707,45 @@
       </c>
       <c r="E26" s="6" t="inlineStr">
         <is>
-          <t>1차 매수선까지 20.6%</t>
+          <t>1차 매수선까지 17.4%</t>
         </is>
       </c>
       <c r="F26" s="7" t="n">
-        <v>442500</v>
+        <v>433500</v>
       </c>
       <c r="G26" s="7" t="n">
-        <v>434500</v>
+        <v>427500</v>
       </c>
       <c r="H26" s="7" t="n">
-        <v>444500</v>
+        <v>439000</v>
       </c>
       <c r="I26" s="7" t="n">
-        <v>458125</v>
+        <v>461075</v>
       </c>
       <c r="J26" s="7" t="n">
-        <v>366500</v>
+        <v>368860</v>
       </c>
       <c r="K26" s="7" t="n">
-        <v>367000</v>
+        <v>369360</v>
       </c>
       <c r="L26" s="8" t="n">
-        <v>0.2057220708446867</v>
+        <v>0.173651721897336</v>
       </c>
       <c r="M26" s="9" t="inlineStr"/>
       <c r="N26" s="9" t="inlineStr"/>
       <c r="O26" s="7" t="n">
-        <v>330300</v>
+        <v>332424</v>
       </c>
       <c r="P26" s="8" t="n">
-        <v>0.3396911898274296</v>
+        <v>0.3040574687748177</v>
       </c>
       <c r="Q26" s="9" t="inlineStr"/>
       <c r="R26" s="9" t="inlineStr"/>
       <c r="S26" s="7" t="n">
-        <v>297270</v>
+        <v>299181.6</v>
       </c>
       <c r="T26" s="8" t="n">
-        <v>0.4885457664749218</v>
+        <v>0.4489527430831306</v>
       </c>
       <c r="U26" s="9" t="inlineStr"/>
       <c r="V26" s="9" t="inlineStr"/>
@@ -2759,7 +2759,7 @@
       <c r="AD26" s="9" t="inlineStr"/>
       <c r="AE26" s="10" t="inlineStr">
         <is>
-          <t>2025-10-14 00:22:53</t>
+          <t>2025-10-16 03:37:11</t>
         </is>
       </c>
       <c r="AF26" s="11" t="n">
@@ -2786,50 +2786,50 @@
       </c>
       <c r="D27" s="5" t="inlineStr">
         <is>
-          <t>WATCHING</t>
+          <t>READY_BUY1</t>
         </is>
       </c>
       <c r="E27" s="6" t="inlineStr">
         <is>
-          <t>1차 매수선까지 11.6%</t>
+          <t>1차 매수선까지 8.2% (접근 중!)</t>
         </is>
       </c>
       <c r="F27" s="7" t="n">
-        <v>23100</v>
+        <v>22250</v>
       </c>
       <c r="G27" s="7" t="n">
-        <v>22800</v>
+        <v>21700</v>
       </c>
       <c r="H27" s="7" t="n">
-        <v>24150</v>
+        <v>22600</v>
       </c>
       <c r="I27" s="7" t="n">
-        <v>25800</v>
+        <v>25640</v>
       </c>
       <c r="J27" s="7" t="n">
-        <v>20640</v>
+        <v>20512</v>
       </c>
       <c r="K27" s="7" t="n">
-        <v>20690</v>
+        <v>20562</v>
       </c>
       <c r="L27" s="8" t="n">
-        <v>0.1164813919768004</v>
+        <v>0.08209318159712091</v>
       </c>
       <c r="M27" s="9" t="inlineStr"/>
       <c r="N27" s="9" t="inlineStr"/>
       <c r="O27" s="7" t="n">
-        <v>18621</v>
+        <v>18505.8</v>
       </c>
       <c r="P27" s="8" t="n">
-        <v>0.2405348799742227</v>
+        <v>0.2023257573301344</v>
       </c>
       <c r="Q27" s="9" t="inlineStr"/>
       <c r="R27" s="9" t="inlineStr"/>
       <c r="S27" s="7" t="n">
-        <v>16758.9</v>
+        <v>16655.22</v>
       </c>
       <c r="T27" s="8" t="n">
-        <v>0.3783720888602473</v>
+        <v>0.3359175081445936</v>
       </c>
       <c r="U27" s="9" t="inlineStr"/>
       <c r="V27" s="9" t="inlineStr"/>
@@ -2843,7 +2843,7 @@
       <c r="AD27" s="9" t="inlineStr"/>
       <c r="AE27" s="10" t="inlineStr">
         <is>
-          <t>2025-10-14 00:22:54</t>
+          <t>2025-10-16 03:37:11</t>
         </is>
       </c>
       <c r="AF27" s="11" t="n">
@@ -2875,45 +2875,45 @@
       </c>
       <c r="E28" s="6" t="inlineStr">
         <is>
-          <t>1차 매수선까지 8.8% (접근 중!)</t>
+          <t>1차 매수선까지 6.3% (접근 중!)</t>
         </is>
       </c>
       <c r="F28" s="7" t="n">
-        <v>25300</v>
+        <v>24200</v>
       </c>
       <c r="G28" s="7" t="n">
-        <v>24750</v>
+        <v>23350</v>
       </c>
       <c r="H28" s="7" t="n">
-        <v>26700</v>
+        <v>24500</v>
       </c>
       <c r="I28" s="7" t="n">
-        <v>29005</v>
+        <v>28395</v>
       </c>
       <c r="J28" s="7" t="n">
-        <v>23204</v>
+        <v>22716</v>
       </c>
       <c r="K28" s="7" t="n">
-        <v>23254</v>
+        <v>22766</v>
       </c>
       <c r="L28" s="8" t="n">
-        <v>0.0879848628192999</v>
+        <v>0.06298866731090222</v>
       </c>
       <c r="M28" s="9" t="inlineStr"/>
       <c r="N28" s="9" t="inlineStr"/>
       <c r="O28" s="7" t="n">
-        <v>20928.6</v>
+        <v>20489.4</v>
       </c>
       <c r="P28" s="8" t="n">
-        <v>0.208872069799222</v>
+        <v>0.1810985192343357</v>
       </c>
       <c r="Q28" s="9" t="inlineStr"/>
       <c r="R28" s="9" t="inlineStr"/>
       <c r="S28" s="7" t="n">
-        <v>18835.74</v>
+        <v>18440.46</v>
       </c>
       <c r="T28" s="8" t="n">
-        <v>0.3431911886658023</v>
+        <v>0.3123316880381507</v>
       </c>
       <c r="U28" s="9" t="inlineStr"/>
       <c r="V28" s="9" t="inlineStr"/>
@@ -2927,7 +2927,7 @@
       <c r="AD28" s="9" t="inlineStr"/>
       <c r="AE28" s="10" t="inlineStr">
         <is>
-          <t>2025-10-14 00:22:54</t>
+          <t>2025-10-16 03:37:11</t>
         </is>
       </c>
       <c r="AF28" s="11" t="n">
@@ -2959,45 +2959,45 @@
       </c>
       <c r="E29" s="6" t="inlineStr">
         <is>
-          <t>1차 매수선까지 12.7%</t>
+          <t>1차 매수선까지 15.4%</t>
         </is>
       </c>
       <c r="F29" s="7" t="n">
-        <v>20400</v>
+        <v>20450</v>
       </c>
       <c r="G29" s="7" t="n">
-        <v>20100</v>
+        <v>19620</v>
       </c>
       <c r="H29" s="7" t="n">
-        <v>21250</v>
+        <v>20500</v>
       </c>
       <c r="I29" s="7" t="n">
-        <v>22555</v>
+        <v>22097</v>
       </c>
       <c r="J29" s="7" t="n">
-        <v>18044</v>
+        <v>17677.6</v>
       </c>
       <c r="K29" s="7" t="n">
-        <v>18094</v>
+        <v>17727.6</v>
       </c>
       <c r="L29" s="8" t="n">
-        <v>0.1274455620647729</v>
+        <v>0.1535684469414922</v>
       </c>
       <c r="M29" s="9" t="inlineStr"/>
       <c r="N29" s="9" t="inlineStr"/>
       <c r="O29" s="7" t="n">
-        <v>16284.6</v>
+        <v>15954.84</v>
       </c>
       <c r="P29" s="8" t="n">
-        <v>0.2527172911830809</v>
+        <v>0.2817427188238802</v>
       </c>
       <c r="Q29" s="9" t="inlineStr"/>
       <c r="R29" s="9" t="inlineStr"/>
       <c r="S29" s="7" t="n">
-        <v>14656.14</v>
+        <v>14359.356</v>
       </c>
       <c r="T29" s="8" t="n">
-        <v>0.3919081013145343</v>
+        <v>0.424158576470978</v>
       </c>
       <c r="U29" s="9" t="inlineStr"/>
       <c r="V29" s="9" t="inlineStr"/>
@@ -3011,7 +3011,7 @@
       <c r="AD29" s="9" t="inlineStr"/>
       <c r="AE29" s="10" t="inlineStr">
         <is>
-          <t>2025-10-14 00:22:54</t>
+          <t>2025-10-16 03:37:12</t>
         </is>
       </c>
       <c r="AF29" s="11" t="n">
@@ -3038,50 +3038,50 @@
       </c>
       <c r="D30" s="5" t="inlineStr">
         <is>
-          <t>WATCHING</t>
+          <t>READY_BUY1</t>
         </is>
       </c>
       <c r="E30" s="6" t="inlineStr">
         <is>
-          <t>1차 매수선까지 12.2%</t>
+          <t>1차 매수선까지 8.4% (접근 중!)</t>
         </is>
       </c>
       <c r="F30" s="7" t="n">
-        <v>49900</v>
+        <v>47750</v>
       </c>
       <c r="G30" s="7" t="n">
-        <v>49600</v>
+        <v>45600</v>
       </c>
       <c r="H30" s="7" t="n">
-        <v>51900</v>
+        <v>47850</v>
       </c>
       <c r="I30" s="7" t="n">
-        <v>55542.5</v>
+        <v>55005</v>
       </c>
       <c r="J30" s="7" t="n">
-        <v>44434</v>
+        <v>44004</v>
       </c>
       <c r="K30" s="7" t="n">
-        <v>44484</v>
+        <v>44054</v>
       </c>
       <c r="L30" s="8" t="n">
-        <v>0.1217516410394749</v>
+        <v>0.08389703545648523</v>
       </c>
       <c r="M30" s="9" t="inlineStr"/>
       <c r="N30" s="9" t="inlineStr"/>
       <c r="O30" s="7" t="n">
-        <v>40035.6</v>
+        <v>39648.6</v>
       </c>
       <c r="P30" s="8" t="n">
-        <v>0.2463907122660832</v>
+        <v>0.2043300393960947</v>
       </c>
       <c r="Q30" s="9" t="inlineStr"/>
       <c r="R30" s="9" t="inlineStr"/>
       <c r="S30" s="7" t="n">
-        <v>36032.04</v>
+        <v>35683.74</v>
       </c>
       <c r="T30" s="8" t="n">
-        <v>0.3848785691845368</v>
+        <v>0.338144488217883</v>
       </c>
       <c r="U30" s="9" t="inlineStr"/>
       <c r="V30" s="9" t="inlineStr"/>
@@ -3095,7 +3095,7 @@
       <c r="AD30" s="9" t="inlineStr"/>
       <c r="AE30" s="10" t="inlineStr">
         <is>
-          <t>2025-10-14 00:22:55</t>
+          <t>2025-10-16 03:37:12</t>
         </is>
       </c>
       <c r="AF30" s="11" t="n">
@@ -3127,45 +3127,45 @@
       </c>
       <c r="E31" s="6" t="inlineStr">
         <is>
-          <t>1차 매수선까지 31.8%</t>
+          <t>1차 매수선까지 31.6%</t>
         </is>
       </c>
       <c r="F31" s="7" t="n">
-        <v>47200</v>
+        <v>47250</v>
       </c>
       <c r="G31" s="7" t="n">
-        <v>46500</v>
+        <v>44050</v>
       </c>
       <c r="H31" s="7" t="n">
-        <v>48950</v>
+        <v>47900</v>
       </c>
       <c r="I31" s="7" t="n">
-        <v>44705</v>
+        <v>44825</v>
       </c>
       <c r="J31" s="7" t="n">
-        <v>35764</v>
+        <v>35860</v>
       </c>
       <c r="K31" s="7" t="n">
-        <v>35814</v>
+        <v>35910</v>
       </c>
       <c r="L31" s="8" t="n">
-        <v>0.3179203663371866</v>
+        <v>0.3157894736842105</v>
       </c>
       <c r="M31" s="9" t="inlineStr"/>
       <c r="N31" s="9" t="inlineStr"/>
       <c r="O31" s="7" t="n">
-        <v>32232.6</v>
+        <v>32319</v>
       </c>
       <c r="P31" s="8" t="n">
-        <v>0.4643559625968738</v>
+        <v>0.4619883040935672</v>
       </c>
       <c r="Q31" s="9" t="inlineStr"/>
       <c r="R31" s="9" t="inlineStr"/>
       <c r="S31" s="7" t="n">
-        <v>29009.34</v>
+        <v>29087.1</v>
       </c>
       <c r="T31" s="8" t="n">
-        <v>0.6270621806631931</v>
+        <v>0.6244314489928524</v>
       </c>
       <c r="U31" s="9" t="inlineStr"/>
       <c r="V31" s="9" t="inlineStr"/>
@@ -3179,7 +3179,7 @@
       <c r="AD31" s="9" t="inlineStr"/>
       <c r="AE31" s="10" t="inlineStr">
         <is>
-          <t>2025-10-14 00:22:55</t>
+          <t>2025-10-16 03:37:12</t>
         </is>
       </c>
       <c r="AF31" s="11" t="n">
@@ -3211,45 +3211,45 @@
       </c>
       <c r="E32" s="6" t="inlineStr">
         <is>
-          <t>1차 매수선까지 10.7%</t>
+          <t>1차 매수선까지 10.4%</t>
         </is>
       </c>
       <c r="F32" s="7" t="n">
-        <v>24000</v>
+        <v>23350</v>
       </c>
       <c r="G32" s="7" t="n">
-        <v>23900</v>
+        <v>22600</v>
       </c>
       <c r="H32" s="7" t="n">
-        <v>24850</v>
+        <v>23450</v>
       </c>
       <c r="I32" s="7" t="n">
-        <v>27045</v>
+        <v>26367.5</v>
       </c>
       <c r="J32" s="7" t="n">
-        <v>21636</v>
+        <v>21094</v>
       </c>
       <c r="K32" s="7" t="n">
-        <v>21686</v>
+        <v>21144</v>
       </c>
       <c r="L32" s="8" t="n">
-        <v>0.1067047864982016</v>
+        <v>0.1043321982595535</v>
       </c>
       <c r="M32" s="9" t="inlineStr"/>
       <c r="N32" s="9" t="inlineStr"/>
       <c r="O32" s="7" t="n">
-        <v>19517.4</v>
+        <v>19029.6</v>
       </c>
       <c r="P32" s="8" t="n">
-        <v>0.2296719849980017</v>
+        <v>0.2270357758439483</v>
       </c>
       <c r="Q32" s="9" t="inlineStr"/>
       <c r="R32" s="9" t="inlineStr"/>
       <c r="S32" s="7" t="n">
-        <v>17565.66</v>
+        <v>17126.64</v>
       </c>
       <c r="T32" s="8" t="n">
-        <v>0.366302205553335</v>
+        <v>0.3633730842710536</v>
       </c>
       <c r="U32" s="9" t="inlineStr"/>
       <c r="V32" s="9" t="inlineStr"/>
@@ -3263,7 +3263,7 @@
       <c r="AD32" s="9" t="inlineStr"/>
       <c r="AE32" s="10" t="inlineStr">
         <is>
-          <t>2025-10-14 00:22:55</t>
+          <t>2025-10-16 03:37:13</t>
         </is>
       </c>
       <c r="AF32" s="11" t="n">
@@ -3295,45 +3295,45 @@
       </c>
       <c r="E33" s="6" t="inlineStr">
         <is>
-          <t>1차 매수선까지 27.6%</t>
+          <t>1차 매수선까지 29.8%</t>
         </is>
       </c>
       <c r="F33" s="7" t="n">
-        <v>420000</v>
+        <v>427500</v>
       </c>
       <c r="G33" s="7" t="n">
-        <v>412000</v>
+        <v>407000</v>
       </c>
       <c r="H33" s="7" t="n">
         <v>428500</v>
       </c>
       <c r="I33" s="7" t="n">
-        <v>410725</v>
+        <v>411175</v>
       </c>
       <c r="J33" s="7" t="n">
-        <v>328580</v>
+        <v>328940</v>
       </c>
       <c r="K33" s="7" t="n">
-        <v>329080</v>
+        <v>329440</v>
       </c>
       <c r="L33" s="8" t="n">
-        <v>0.2762854017260241</v>
+        <v>0.297656629431763</v>
       </c>
       <c r="M33" s="9" t="inlineStr"/>
       <c r="N33" s="9" t="inlineStr"/>
       <c r="O33" s="7" t="n">
-        <v>296172</v>
+        <v>296496</v>
       </c>
       <c r="P33" s="8" t="n">
-        <v>0.4180948908066934</v>
+        <v>0.4418406993686255</v>
       </c>
       <c r="Q33" s="9" t="inlineStr"/>
       <c r="R33" s="9" t="inlineStr"/>
       <c r="S33" s="7" t="n">
-        <v>266554.8</v>
+        <v>266846.4</v>
       </c>
       <c r="T33" s="8" t="n">
-        <v>0.5756609897852151</v>
+        <v>0.6020452215206948</v>
       </c>
       <c r="U33" s="9" t="inlineStr"/>
       <c r="V33" s="9" t="inlineStr"/>
@@ -3347,7 +3347,7 @@
       <c r="AD33" s="9" t="inlineStr"/>
       <c r="AE33" s="10" t="inlineStr">
         <is>
-          <t>2025-10-14 00:22:56</t>
+          <t>2025-10-16 03:37:13</t>
         </is>
       </c>
       <c r="AF33" s="11" t="n">
@@ -3379,45 +3379,45 @@
       </c>
       <c r="E34" s="6" t="inlineStr">
         <is>
-          <t>1차 매수선까지 26.5%</t>
+          <t>1차 매수선까지 25.4%</t>
         </is>
       </c>
       <c r="F34" s="7" t="n">
-        <v>202000</v>
+        <v>200500</v>
       </c>
       <c r="G34" s="7" t="n">
-        <v>198400</v>
+        <v>195500</v>
       </c>
       <c r="H34" s="7" t="n">
-        <v>208000</v>
+        <v>203000</v>
       </c>
       <c r="I34" s="7" t="n">
-        <v>198970</v>
+        <v>199280</v>
       </c>
       <c r="J34" s="7" t="n">
-        <v>159176</v>
+        <v>159424</v>
       </c>
       <c r="K34" s="7" t="n">
-        <v>159676</v>
+        <v>159924</v>
       </c>
       <c r="L34" s="8" t="n">
-        <v>0.2650617500438387</v>
+        <v>0.2537205172456917</v>
       </c>
       <c r="M34" s="9" t="inlineStr"/>
       <c r="N34" s="9" t="inlineStr"/>
       <c r="O34" s="7" t="n">
-        <v>143708.4</v>
+        <v>143931.6</v>
       </c>
       <c r="P34" s="8" t="n">
-        <v>0.4056241667153765</v>
+        <v>0.3930227969396574</v>
       </c>
       <c r="Q34" s="9" t="inlineStr"/>
       <c r="R34" s="9" t="inlineStr"/>
       <c r="S34" s="7" t="n">
-        <v>129337.56</v>
+        <v>129538.44</v>
       </c>
       <c r="T34" s="8" t="n">
-        <v>0.5618046296837516</v>
+        <v>0.5478031077107305</v>
       </c>
       <c r="U34" s="9" t="inlineStr"/>
       <c r="V34" s="9" t="inlineStr"/>
@@ -3431,7 +3431,7 @@
       <c r="AD34" s="9" t="inlineStr"/>
       <c r="AE34" s="10" t="inlineStr">
         <is>
-          <t>2025-10-14 00:22:56</t>
+          <t>2025-10-16 03:37:13</t>
         </is>
       </c>
       <c r="AF34" s="11" t="n">
@@ -3463,45 +3463,45 @@
       </c>
       <c r="E35" s="6" t="inlineStr">
         <is>
-          <t>1차 매수선까지 28.0%</t>
+          <t>1차 매수선까지 24.3%</t>
         </is>
       </c>
       <c r="F35" s="7" t="n">
-        <v>22250</v>
+        <v>21650</v>
       </c>
       <c r="G35" s="7" t="n">
-        <v>21850</v>
+        <v>21100</v>
       </c>
       <c r="H35" s="7" t="n">
-        <v>22600</v>
+        <v>21700</v>
       </c>
       <c r="I35" s="7" t="n">
-        <v>21665</v>
+        <v>21710</v>
       </c>
       <c r="J35" s="7" t="n">
-        <v>17332</v>
+        <v>17368</v>
       </c>
       <c r="K35" s="7" t="n">
-        <v>17382</v>
+        <v>17418</v>
       </c>
       <c r="L35" s="8" t="n">
-        <v>0.2800598320101254</v>
+        <v>0.242967045585027</v>
       </c>
       <c r="M35" s="9" t="inlineStr"/>
       <c r="N35" s="9" t="inlineStr"/>
       <c r="O35" s="7" t="n">
-        <v>15643.8</v>
+        <v>15676.2</v>
       </c>
       <c r="P35" s="8" t="n">
-        <v>0.4222887022334726</v>
+        <v>0.3810744950944744</v>
       </c>
       <c r="Q35" s="9" t="inlineStr"/>
       <c r="R35" s="9" t="inlineStr"/>
       <c r="S35" s="7" t="n">
-        <v>14079.42</v>
+        <v>14108.58</v>
       </c>
       <c r="T35" s="8" t="n">
-        <v>0.5803207802594139</v>
+        <v>0.5345272167716381</v>
       </c>
       <c r="U35" s="9" t="inlineStr"/>
       <c r="V35" s="9" t="inlineStr"/>
@@ -3515,7 +3515,7 @@
       <c r="AD35" s="9" t="inlineStr"/>
       <c r="AE35" s="10" t="inlineStr">
         <is>
-          <t>2025-10-14 00:22:56</t>
+          <t>2025-10-16 03:37:14</t>
         </is>
       </c>
       <c r="AF35" s="11" t="n">
@@ -3547,45 +3547,45 @@
       </c>
       <c r="E36" s="6" t="inlineStr">
         <is>
-          <t>1차 매수선까지 30.2%</t>
+          <t>1차 매수선까지 45.9%</t>
         </is>
       </c>
       <c r="F36" s="7" t="n">
-        <v>1446000</v>
+        <v>1649000</v>
       </c>
       <c r="G36" s="7" t="n">
-        <v>1428000</v>
+        <v>1454000</v>
       </c>
       <c r="H36" s="7" t="n">
-        <v>1493000</v>
+        <v>1652000</v>
       </c>
       <c r="I36" s="7" t="n">
-        <v>1387100</v>
+        <v>1411650</v>
       </c>
       <c r="J36" s="7" t="n">
-        <v>1109680</v>
+        <v>1129320</v>
       </c>
       <c r="K36" s="7" t="n">
-        <v>1110680</v>
+        <v>1130320</v>
       </c>
       <c r="L36" s="8" t="n">
-        <v>0.3019051391940073</v>
+        <v>0.4588789015500037</v>
       </c>
       <c r="M36" s="9" t="inlineStr"/>
       <c r="N36" s="9" t="inlineStr"/>
       <c r="O36" s="7" t="n">
-        <v>999612</v>
+        <v>1017288</v>
       </c>
       <c r="P36" s="8" t="n">
-        <v>0.4465612657711192</v>
+        <v>0.6209765572777817</v>
       </c>
       <c r="Q36" s="9" t="inlineStr"/>
       <c r="R36" s="9" t="inlineStr"/>
       <c r="S36" s="7" t="n">
-        <v>899650.8</v>
+        <v>915559.2000000001</v>
       </c>
       <c r="T36" s="8" t="n">
-        <v>0.6072902953012435</v>
+        <v>0.8010850636419795</v>
       </c>
       <c r="U36" s="9" t="inlineStr"/>
       <c r="V36" s="9" t="inlineStr"/>
@@ -3599,7 +3599,7 @@
       <c r="AD36" s="9" t="inlineStr"/>
       <c r="AE36" s="10" t="inlineStr">
         <is>
-          <t>2025-10-14 00:22:57</t>
+          <t>2025-10-16 03:37:14</t>
         </is>
       </c>
       <c r="AF36" s="11" t="n">
@@ -3631,45 +3631,45 @@
       </c>
       <c r="E37" s="6" t="inlineStr">
         <is>
-          <t>1차 매수선까지 16.1%</t>
+          <t>1차 매수선까지 14.9%</t>
         </is>
       </c>
       <c r="F37" s="7" t="n">
-        <v>465000</v>
+        <v>458500</v>
       </c>
       <c r="G37" s="7" t="n">
-        <v>460500</v>
+        <v>446500</v>
       </c>
       <c r="H37" s="7" t="n">
-        <v>476250</v>
+        <v>459000</v>
       </c>
       <c r="I37" s="7" t="n">
-        <v>500050</v>
+        <v>498075</v>
       </c>
       <c r="J37" s="7" t="n">
-        <v>400040</v>
+        <v>398460</v>
       </c>
       <c r="K37" s="7" t="n">
-        <v>400540</v>
+        <v>398960</v>
       </c>
       <c r="L37" s="8" t="n">
-        <v>0.1609327407999201</v>
+        <v>0.1492380188490074</v>
       </c>
       <c r="M37" s="9" t="inlineStr"/>
       <c r="N37" s="9" t="inlineStr"/>
       <c r="O37" s="7" t="n">
-        <v>360486</v>
+        <v>359064</v>
       </c>
       <c r="P37" s="8" t="n">
-        <v>0.2899252675554668</v>
+        <v>0.2769311320544527</v>
       </c>
       <c r="Q37" s="9" t="inlineStr"/>
       <c r="R37" s="9" t="inlineStr"/>
       <c r="S37" s="7" t="n">
-        <v>324437.4</v>
+        <v>323157.6</v>
       </c>
       <c r="T37" s="8" t="n">
-        <v>0.4332502972838519</v>
+        <v>0.4188123689493917</v>
       </c>
       <c r="U37" s="9" t="inlineStr"/>
       <c r="V37" s="9" t="inlineStr"/>
@@ -3683,7 +3683,7 @@
       <c r="AD37" s="9" t="inlineStr"/>
       <c r="AE37" s="10" t="inlineStr">
         <is>
-          <t>2025-10-14 00:22:57</t>
+          <t>2025-10-16 03:37:14</t>
         </is>
       </c>
       <c r="AF37" s="11" t="n">
@@ -3695,7 +3695,7 @@
     <row r="38">
       <c r="A38" s="5" t="inlineStr">
         <is>
-          <t>0008Z0</t>
+          <t>000080</t>
         </is>
       </c>
       <c r="B38" s="5" t="inlineStr">
@@ -3715,45 +3715,45 @@
       </c>
       <c r="E38" s="6" t="inlineStr">
         <is>
-          <t>1차 매수선까지 17.6%</t>
+          <t>1차 매수선까지 22.7%</t>
         </is>
       </c>
       <c r="F38" s="7" t="n">
-        <v>40700</v>
+        <v>18840</v>
       </c>
       <c r="G38" s="7" t="n">
-        <v>40650</v>
+        <v>18750</v>
       </c>
       <c r="H38" s="7" t="n">
-        <v>42650</v>
+        <v>18920</v>
       </c>
       <c r="I38" s="7" t="n">
-        <v>43212.5</v>
+        <v>19126</v>
       </c>
       <c r="J38" s="7" t="n">
-        <v>34570</v>
+        <v>15300.8</v>
       </c>
       <c r="K38" s="7" t="n">
-        <v>34620</v>
+        <v>15350.8</v>
       </c>
       <c r="L38" s="8" t="n">
-        <v>0.1756210283073368</v>
+        <v>0.2272976001250748</v>
       </c>
       <c r="M38" s="9" t="inlineStr"/>
       <c r="N38" s="9" t="inlineStr"/>
       <c r="O38" s="7" t="n">
-        <v>31158</v>
+        <v>13815.72</v>
       </c>
       <c r="P38" s="8" t="n">
-        <v>0.306245587008152</v>
+        <v>0.363664000138972</v>
       </c>
       <c r="Q38" s="9" t="inlineStr"/>
       <c r="R38" s="9" t="inlineStr"/>
       <c r="S38" s="7" t="n">
-        <v>28042.2</v>
+        <v>12434.148</v>
       </c>
       <c r="T38" s="8" t="n">
-        <v>0.4513839855646133</v>
+        <v>0.5151822223766356</v>
       </c>
       <c r="U38" s="9" t="inlineStr"/>
       <c r="V38" s="9" t="inlineStr"/>
@@ -3767,7 +3767,7 @@
       <c r="AD38" s="9" t="inlineStr"/>
       <c r="AE38" s="10" t="inlineStr">
         <is>
-          <t>2025-10-14 00:22:57</t>
+          <t>2025-10-16 03:37:15</t>
         </is>
       </c>
       <c r="AF38" s="11" t="n">
@@ -3799,45 +3799,45 @@
       </c>
       <c r="E39" s="6" t="inlineStr">
         <is>
-          <t>1차 매수선까지 13.6%</t>
+          <t>1차 매수선까지 10.8%</t>
         </is>
       </c>
       <c r="F39" s="7" t="n">
-        <v>17490</v>
+        <v>16900</v>
       </c>
       <c r="G39" s="7" t="n">
-        <v>17210</v>
+        <v>16780</v>
       </c>
       <c r="H39" s="7" t="n">
-        <v>18060</v>
+        <v>17120</v>
       </c>
       <c r="I39" s="7" t="n">
-        <v>19191</v>
+        <v>18997</v>
       </c>
       <c r="J39" s="7" t="n">
-        <v>15352.8</v>
+        <v>15197.6</v>
       </c>
       <c r="K39" s="7" t="n">
-        <v>15402.8</v>
+        <v>15247.6</v>
       </c>
       <c r="L39" s="8" t="n">
-        <v>0.135507829745241</v>
+        <v>0.1083711534930087</v>
       </c>
       <c r="M39" s="9" t="inlineStr"/>
       <c r="N39" s="9" t="inlineStr"/>
       <c r="O39" s="7" t="n">
-        <v>13862.52</v>
+        <v>13722.84</v>
       </c>
       <c r="P39" s="8" t="n">
-        <v>0.2616753663836012</v>
+        <v>0.2315235038811208</v>
       </c>
       <c r="Q39" s="9" t="inlineStr"/>
       <c r="R39" s="9" t="inlineStr"/>
       <c r="S39" s="7" t="n">
-        <v>12476.268</v>
+        <v>12350.556</v>
       </c>
       <c r="T39" s="8" t="n">
-        <v>0.4018615182040014</v>
+        <v>0.3683594487568008</v>
       </c>
       <c r="U39" s="9" t="inlineStr"/>
       <c r="V39" s="9" t="inlineStr"/>
@@ -3851,7 +3851,7 @@
       <c r="AD39" s="9" t="inlineStr"/>
       <c r="AE39" s="10" t="inlineStr">
         <is>
-          <t>2025-10-14 00:22:58</t>
+          <t>2025-10-16 03:37:15</t>
         </is>
       </c>
       <c r="AF39" s="11" t="n">
@@ -3883,45 +3883,45 @@
       </c>
       <c r="E40" s="6" t="inlineStr">
         <is>
-          <t>1차 매수선까지 14.7%</t>
+          <t>1차 매수선까지 15.0%</t>
         </is>
       </c>
       <c r="F40" s="7" t="n">
-        <v>91500</v>
+        <v>90400</v>
       </c>
       <c r="G40" s="7" t="n">
-        <v>90600</v>
+        <v>88600</v>
       </c>
       <c r="H40" s="7" t="n">
-        <v>94400</v>
+        <v>91100</v>
       </c>
       <c r="I40" s="7" t="n">
-        <v>99630</v>
+        <v>98165</v>
       </c>
       <c r="J40" s="7" t="n">
-        <v>79704</v>
+        <v>78532</v>
       </c>
       <c r="K40" s="7" t="n">
-        <v>79804</v>
+        <v>78632</v>
       </c>
       <c r="L40" s="8" t="n">
-        <v>0.146559069720816</v>
+        <v>0.1496591718384373</v>
       </c>
       <c r="M40" s="9" t="inlineStr"/>
       <c r="N40" s="9" t="inlineStr"/>
       <c r="O40" s="7" t="n">
-        <v>71823.60000000001</v>
+        <v>70768.8</v>
       </c>
       <c r="P40" s="8" t="n">
-        <v>0.2739545219120177</v>
+        <v>0.2773990798204859</v>
       </c>
       <c r="Q40" s="9" t="inlineStr"/>
       <c r="R40" s="9" t="inlineStr"/>
       <c r="S40" s="7" t="n">
-        <v>64641.24000000001</v>
+        <v>63691.92000000001</v>
       </c>
       <c r="T40" s="8" t="n">
-        <v>0.4155050243466863</v>
+        <v>0.4193323109116507</v>
       </c>
       <c r="U40" s="9" t="inlineStr"/>
       <c r="V40" s="9" t="inlineStr"/>
@@ -3935,7 +3935,7 @@
       <c r="AD40" s="9" t="inlineStr"/>
       <c r="AE40" s="10" t="inlineStr">
         <is>
-          <t>2025-10-14 00:22:58</t>
+          <t>2025-10-16 03:37:16</t>
         </is>
       </c>
       <c r="AF40" s="11" t="n">
@@ -3967,45 +3967,45 @@
       </c>
       <c r="E41" s="6" t="inlineStr">
         <is>
-          <t>1차 매수선까지 40.4%</t>
+          <t>1차 매수선까지 32.0%</t>
         </is>
       </c>
       <c r="F41" s="7" t="n">
-        <v>15190</v>
+        <v>14580</v>
       </c>
       <c r="G41" s="7" t="n">
-        <v>15050</v>
+        <v>14070</v>
       </c>
       <c r="H41" s="7" t="n">
-        <v>15450</v>
+        <v>14730</v>
       </c>
       <c r="I41" s="7" t="n">
-        <v>13460.5</v>
+        <v>13742.5</v>
       </c>
       <c r="J41" s="7" t="n">
-        <v>10768.4</v>
+        <v>10994</v>
       </c>
       <c r="K41" s="7" t="n">
-        <v>10818.4</v>
+        <v>11044</v>
       </c>
       <c r="L41" s="8" t="n">
-        <v>0.4040893292908376</v>
+        <v>0.3201738500543281</v>
       </c>
       <c r="M41" s="9" t="inlineStr"/>
       <c r="N41" s="9" t="inlineStr"/>
       <c r="O41" s="7" t="n">
-        <v>9736.560000000001</v>
+        <v>9939.6</v>
       </c>
       <c r="P41" s="8" t="n">
-        <v>0.5600992547675974</v>
+        <v>0.4668598333936979</v>
       </c>
       <c r="Q41" s="9" t="inlineStr"/>
       <c r="R41" s="9" t="inlineStr"/>
       <c r="S41" s="7" t="n">
-        <v>8762.904000000002</v>
+        <v>8945.640000000001</v>
       </c>
       <c r="T41" s="8" t="n">
-        <v>0.7334436164084415</v>
+        <v>0.6298442593263308</v>
       </c>
       <c r="U41" s="9" t="inlineStr"/>
       <c r="V41" s="9" t="inlineStr"/>
@@ -4019,7 +4019,7 @@
       <c r="AD41" s="9" t="inlineStr"/>
       <c r="AE41" s="10" t="inlineStr">
         <is>
-          <t>2025-10-14 00:22:58</t>
+          <t>2025-10-16 03:37:16</t>
         </is>
       </c>
       <c r="AF41" s="11" t="n">
@@ -4051,45 +4051,45 @@
       </c>
       <c r="E42" s="6" t="inlineStr">
         <is>
-          <t>1차 매수선까지 21.9%</t>
+          <t>1차 매수선까지 34.5%</t>
         </is>
       </c>
       <c r="F42" s="7" t="n">
-        <v>35700</v>
+        <v>39450</v>
       </c>
       <c r="G42" s="7" t="n">
-        <v>35100</v>
+        <v>37100</v>
       </c>
       <c r="H42" s="7" t="n">
-        <v>36100</v>
+        <v>39550</v>
       </c>
       <c r="I42" s="7" t="n">
-        <v>36552.5</v>
+        <v>36595</v>
       </c>
       <c r="J42" s="7" t="n">
-        <v>29242</v>
+        <v>29276</v>
       </c>
       <c r="K42" s="7" t="n">
-        <v>29292</v>
+        <v>29326</v>
       </c>
       <c r="L42" s="8" t="n">
-        <v>0.2187628021302745</v>
+        <v>0.3452226693036896</v>
       </c>
       <c r="M42" s="9" t="inlineStr"/>
       <c r="N42" s="9" t="inlineStr"/>
       <c r="O42" s="7" t="n">
-        <v>26362.8</v>
+        <v>26393.4</v>
       </c>
       <c r="P42" s="8" t="n">
-        <v>0.3541808912558606</v>
+        <v>0.4946918547818772</v>
       </c>
       <c r="Q42" s="9" t="inlineStr"/>
       <c r="R42" s="9" t="inlineStr"/>
       <c r="S42" s="7" t="n">
-        <v>23726.52</v>
+        <v>23754.06</v>
       </c>
       <c r="T42" s="8" t="n">
-        <v>0.5046454347287339</v>
+        <v>0.6607687275354192</v>
       </c>
       <c r="U42" s="9" t="inlineStr"/>
       <c r="V42" s="9" t="inlineStr"/>
@@ -4103,7 +4103,7 @@
       <c r="AD42" s="9" t="inlineStr"/>
       <c r="AE42" s="10" t="inlineStr">
         <is>
-          <t>2025-10-14 00:22:59</t>
+          <t>2025-10-16 03:37:16</t>
         </is>
       </c>
       <c r="AF42" s="11" t="n">
@@ -4135,45 +4135,45 @@
       </c>
       <c r="E43" s="6" t="inlineStr">
         <is>
-          <t>1차 매수선까지 21.4%</t>
+          <t>1차 매수선까지 19.1%</t>
         </is>
       </c>
       <c r="F43" s="7" t="n">
-        <v>78800</v>
+        <v>77000</v>
       </c>
       <c r="G43" s="7" t="n">
-        <v>77500</v>
+        <v>75300</v>
       </c>
       <c r="H43" s="7" t="n">
-        <v>79800</v>
+        <v>77600</v>
       </c>
       <c r="I43" s="7" t="n">
-        <v>81035</v>
+        <v>80720</v>
       </c>
       <c r="J43" s="7" t="n">
-        <v>64828</v>
+        <v>64576</v>
       </c>
       <c r="K43" s="7" t="n">
-        <v>64928</v>
+        <v>64676</v>
       </c>
       <c r="L43" s="8" t="n">
-        <v>0.2136520453425333</v>
+        <v>0.1905498175521059</v>
       </c>
       <c r="M43" s="9" t="inlineStr"/>
       <c r="N43" s="9" t="inlineStr"/>
       <c r="O43" s="7" t="n">
-        <v>58435.2</v>
+        <v>58208.4</v>
       </c>
       <c r="P43" s="8" t="n">
-        <v>0.3485022726028146</v>
+        <v>0.3228331306134509</v>
       </c>
       <c r="Q43" s="9" t="inlineStr"/>
       <c r="R43" s="9" t="inlineStr"/>
       <c r="S43" s="7" t="n">
-        <v>52591.68000000001</v>
+        <v>52387.56</v>
       </c>
       <c r="T43" s="8" t="n">
-        <v>0.4983358584475717</v>
+        <v>0.4698145895705009</v>
       </c>
       <c r="U43" s="9" t="inlineStr"/>
       <c r="V43" s="9" t="inlineStr"/>
@@ -4187,7 +4187,7 @@
       <c r="AD43" s="9" t="inlineStr"/>
       <c r="AE43" s="10" t="inlineStr">
         <is>
-          <t>2025-10-14 00:22:59</t>
+          <t>2025-10-16 03:37:17</t>
         </is>
       </c>
       <c r="AF43" s="11" t="n">
@@ -4219,45 +4219,45 @@
       </c>
       <c r="E44" s="6" t="inlineStr">
         <is>
-          <t>1차 매수선까지 39.5%</t>
+          <t>1차 매수선까지 32.9%</t>
         </is>
       </c>
       <c r="F44" s="7" t="n">
-        <v>259000</v>
+        <v>249000</v>
       </c>
       <c r="G44" s="7" t="n">
-        <v>250500</v>
+        <v>245000</v>
       </c>
       <c r="H44" s="7" t="n">
-        <v>263500</v>
+        <v>251500</v>
       </c>
       <c r="I44" s="7" t="n">
-        <v>231425</v>
+        <v>233650</v>
       </c>
       <c r="J44" s="7" t="n">
-        <v>185140</v>
+        <v>186920</v>
       </c>
       <c r="K44" s="7" t="n">
-        <v>185640</v>
+        <v>187420</v>
       </c>
       <c r="L44" s="8" t="n">
-        <v>0.3951734539969834</v>
+        <v>0.3285668551915484</v>
       </c>
       <c r="M44" s="9" t="inlineStr"/>
       <c r="N44" s="9" t="inlineStr"/>
       <c r="O44" s="7" t="n">
-        <v>167076</v>
+        <v>168678</v>
       </c>
       <c r="P44" s="8" t="n">
-        <v>0.5501927266633149</v>
+        <v>0.476185394657276</v>
       </c>
       <c r="Q44" s="9" t="inlineStr"/>
       <c r="R44" s="9" t="inlineStr"/>
       <c r="S44" s="7" t="n">
-        <v>150368.4</v>
+        <v>151810.2</v>
       </c>
       <c r="T44" s="8" t="n">
-        <v>0.722436362959239</v>
+        <v>0.6402059940636399</v>
       </c>
       <c r="U44" s="9" t="inlineStr"/>
       <c r="V44" s="9" t="inlineStr"/>
@@ -4271,7 +4271,7 @@
       <c r="AD44" s="9" t="inlineStr"/>
       <c r="AE44" s="10" t="inlineStr">
         <is>
-          <t>2025-10-14 00:22:59</t>
+          <t>2025-10-16 03:37:17</t>
         </is>
       </c>
       <c r="AF44" s="11" t="n">
@@ -4303,45 +4303,45 @@
       </c>
       <c r="E45" s="6" t="inlineStr">
         <is>
-          <t>1차 매수선까지 19.3%</t>
+          <t>1차 매수선까지 19.5%</t>
         </is>
       </c>
       <c r="F45" s="7" t="n">
-        <v>102400</v>
+        <v>102000</v>
       </c>
       <c r="G45" s="7" t="n">
-        <v>101050</v>
+        <v>101200</v>
       </c>
       <c r="H45" s="7" t="n">
-        <v>103700</v>
+        <v>102500</v>
       </c>
       <c r="I45" s="7" t="n">
-        <v>107145</v>
+        <v>106530</v>
       </c>
       <c r="J45" s="7" t="n">
-        <v>85716</v>
+        <v>85224</v>
       </c>
       <c r="K45" s="7" t="n">
-        <v>85816</v>
+        <v>85324</v>
       </c>
       <c r="L45" s="8" t="n">
-        <v>0.1932506758646406</v>
+        <v>0.1954432516056444</v>
       </c>
       <c r="M45" s="9" t="inlineStr"/>
       <c r="N45" s="9" t="inlineStr"/>
       <c r="O45" s="7" t="n">
-        <v>77234.40000000001</v>
+        <v>76791.60000000001</v>
       </c>
       <c r="P45" s="8" t="n">
-        <v>0.325834084294045</v>
+        <v>0.328270279561827</v>
       </c>
       <c r="Q45" s="9" t="inlineStr"/>
       <c r="R45" s="9" t="inlineStr"/>
       <c r="S45" s="7" t="n">
-        <v>69510.96000000001</v>
+        <v>69112.44</v>
       </c>
       <c r="T45" s="8" t="n">
-        <v>0.4731489825489389</v>
+        <v>0.4758558661798078</v>
       </c>
       <c r="U45" s="9" t="inlineStr"/>
       <c r="V45" s="9" t="inlineStr"/>
@@ -4355,7 +4355,7 @@
       <c r="AD45" s="9" t="inlineStr"/>
       <c r="AE45" s="10" t="inlineStr">
         <is>
-          <t>2025-10-14 00:23:00</t>
+          <t>2025-10-16 03:37:17</t>
         </is>
       </c>
       <c r="AF45" s="11" t="n">
@@ -4387,45 +4387,45 @@
       </c>
       <c r="E46" s="6" t="inlineStr">
         <is>
-          <t>1차 매수선까지 25.1%</t>
+          <t>1차 매수선까지 32.3%</t>
         </is>
       </c>
       <c r="F46" s="7" t="n">
-        <v>117800</v>
+        <v>125400</v>
       </c>
       <c r="G46" s="7" t="n">
-        <v>109500</v>
+        <v>121400</v>
       </c>
       <c r="H46" s="7" t="n">
-        <v>119700</v>
+        <v>126700</v>
       </c>
       <c r="I46" s="7" t="n">
-        <v>117560</v>
+        <v>118385</v>
       </c>
       <c r="J46" s="7" t="n">
-        <v>94048</v>
+        <v>94708</v>
       </c>
       <c r="K46" s="7" t="n">
-        <v>94148</v>
+        <v>94808</v>
       </c>
       <c r="L46" s="8" t="n">
-        <v>0.2512214810723541</v>
+        <v>0.3226731921356848</v>
       </c>
       <c r="M46" s="9" t="inlineStr"/>
       <c r="N46" s="9" t="inlineStr"/>
       <c r="O46" s="7" t="n">
-        <v>84733.2</v>
+        <v>85327.2</v>
       </c>
       <c r="P46" s="8" t="n">
-        <v>0.3902460900803936</v>
+        <v>0.4696368801507609</v>
       </c>
       <c r="Q46" s="9" t="inlineStr"/>
       <c r="R46" s="9" t="inlineStr"/>
       <c r="S46" s="7" t="n">
-        <v>76259.88</v>
+        <v>76794.48</v>
       </c>
       <c r="T46" s="8" t="n">
-        <v>0.5447178778671038</v>
+        <v>0.6329298668341788</v>
       </c>
       <c r="U46" s="9" t="inlineStr"/>
       <c r="V46" s="9" t="inlineStr"/>
@@ -4439,7 +4439,7 @@
       <c r="AD46" s="9" t="inlineStr"/>
       <c r="AE46" s="10" t="inlineStr">
         <is>
-          <t>2025-10-14 00:23:00</t>
+          <t>2025-10-16 03:37:18</t>
         </is>
       </c>
       <c r="AF46" s="11" t="n">
@@ -4471,45 +4471,45 @@
       </c>
       <c r="E47" s="6" t="inlineStr">
         <is>
-          <t>1차 매수선까지 28.0%</t>
+          <t>1차 매수선까지 32.8%</t>
         </is>
       </c>
       <c r="F47" s="7" t="n">
-        <v>210500</v>
+        <v>221000</v>
       </c>
       <c r="G47" s="7" t="n">
-        <v>201500</v>
+        <v>217500</v>
       </c>
       <c r="H47" s="7" t="n">
-        <v>214000</v>
+        <v>223500</v>
       </c>
       <c r="I47" s="7" t="n">
-        <v>204920</v>
+        <v>207470</v>
       </c>
       <c r="J47" s="7" t="n">
-        <v>163936</v>
+        <v>165976</v>
       </c>
       <c r="K47" s="7" t="n">
-        <v>164436</v>
+        <v>166476</v>
       </c>
       <c r="L47" s="8" t="n">
-        <v>0.2801333041426452</v>
+        <v>0.327518681371489</v>
       </c>
       <c r="M47" s="9" t="inlineStr"/>
       <c r="N47" s="9" t="inlineStr"/>
       <c r="O47" s="7" t="n">
-        <v>147992.4</v>
+        <v>149828.4</v>
       </c>
       <c r="P47" s="8" t="n">
-        <v>0.4223703379362724</v>
+        <v>0.4750207570794323</v>
       </c>
       <c r="Q47" s="9" t="inlineStr"/>
       <c r="R47" s="9" t="inlineStr"/>
       <c r="S47" s="7" t="n">
-        <v>133193.16</v>
+        <v>134845.56</v>
       </c>
       <c r="T47" s="8" t="n">
-        <v>0.5804114865958582</v>
+        <v>0.6389119523104803</v>
       </c>
       <c r="U47" s="9" t="inlineStr"/>
       <c r="V47" s="9" t="inlineStr"/>
@@ -4523,7 +4523,7 @@
       <c r="AD47" s="9" t="inlineStr"/>
       <c r="AE47" s="10" t="inlineStr">
         <is>
-          <t>2025-10-14 00:23:00</t>
+          <t>2025-10-16 03:37:18</t>
         </is>
       </c>
       <c r="AF47" s="11" t="n">
@@ -4555,45 +4555,45 @@
       </c>
       <c r="E48" s="6" t="inlineStr">
         <is>
-          <t>1차 매수선까지 20.4%</t>
+          <t>1차 매수선까지 16.1%</t>
         </is>
       </c>
       <c r="F48" s="7" t="n">
-        <v>993000</v>
+        <v>956000</v>
       </c>
       <c r="G48" s="7" t="n">
-        <v>991000</v>
+        <v>923000</v>
       </c>
       <c r="H48" s="7" t="n">
-        <v>1045000</v>
+        <v>969000</v>
       </c>
       <c r="I48" s="7" t="n">
-        <v>1029700</v>
+        <v>1028250</v>
       </c>
       <c r="J48" s="7" t="n">
-        <v>823760</v>
+        <v>822600</v>
       </c>
       <c r="K48" s="7" t="n">
-        <v>824760</v>
+        <v>823600</v>
       </c>
       <c r="L48" s="8" t="n">
-        <v>0.2039866142877928</v>
+        <v>0.1607576493443419</v>
       </c>
       <c r="M48" s="9" t="inlineStr"/>
       <c r="N48" s="9" t="inlineStr"/>
       <c r="O48" s="7" t="n">
-        <v>742284</v>
+        <v>741240</v>
       </c>
       <c r="P48" s="8" t="n">
-        <v>0.3377629047642142</v>
+        <v>0.2897307214937133</v>
       </c>
       <c r="Q48" s="9" t="inlineStr"/>
       <c r="R48" s="9" t="inlineStr"/>
       <c r="S48" s="7" t="n">
-        <v>668055.6</v>
+        <v>667116</v>
       </c>
       <c r="T48" s="8" t="n">
-        <v>0.4864032275157936</v>
+        <v>0.4330341349930147</v>
       </c>
       <c r="U48" s="9" t="inlineStr"/>
       <c r="V48" s="9" t="inlineStr"/>
@@ -4607,7 +4607,7 @@
       <c r="AD48" s="9" t="inlineStr"/>
       <c r="AE48" s="10" t="inlineStr">
         <is>
-          <t>2025-10-14 00:23:01</t>
+          <t>2025-10-16 03:37:18</t>
         </is>
       </c>
       <c r="AF48" s="11" t="n">
@@ -4639,45 +4639,45 @@
       </c>
       <c r="E49" s="6" t="inlineStr">
         <is>
-          <t>1차 매수선까지 25.2%</t>
+          <t>1차 매수선까지 28.1%</t>
         </is>
       </c>
       <c r="F49" s="7" t="n">
-        <v>218500</v>
+        <v>224000</v>
       </c>
       <c r="G49" s="7" t="n">
-        <v>214000</v>
+        <v>220000</v>
       </c>
       <c r="H49" s="7" t="n">
-        <v>219500</v>
+        <v>224000</v>
       </c>
       <c r="I49" s="7" t="n">
-        <v>217575</v>
+        <v>217975</v>
       </c>
       <c r="J49" s="7" t="n">
-        <v>174060</v>
+        <v>174380</v>
       </c>
       <c r="K49" s="7" t="n">
-        <v>174560</v>
+        <v>174880</v>
       </c>
       <c r="L49" s="8" t="n">
-        <v>0.2517186067827681</v>
+        <v>0.2808783165599268</v>
       </c>
       <c r="M49" s="9" t="inlineStr"/>
       <c r="N49" s="9" t="inlineStr"/>
       <c r="O49" s="7" t="n">
-        <v>157104</v>
+        <v>157392</v>
       </c>
       <c r="P49" s="8" t="n">
-        <v>0.3907984519808534</v>
+        <v>0.4231981295110298</v>
       </c>
       <c r="Q49" s="9" t="inlineStr"/>
       <c r="R49" s="9" t="inlineStr"/>
       <c r="S49" s="7" t="n">
-        <v>141393.6</v>
+        <v>141652.8</v>
       </c>
       <c r="T49" s="8" t="n">
-        <v>0.5453316133120594</v>
+        <v>0.581331255012255</v>
       </c>
       <c r="U49" s="9" t="inlineStr"/>
       <c r="V49" s="9" t="inlineStr"/>
@@ -4691,7 +4691,7 @@
       <c r="AD49" s="9" t="inlineStr"/>
       <c r="AE49" s="10" t="inlineStr">
         <is>
-          <t>2025-10-14 00:23:01</t>
+          <t>2025-10-16 03:37:19</t>
         </is>
       </c>
       <c r="AF49" s="11" t="n">
@@ -4723,45 +4723,45 @@
       </c>
       <c r="E50" s="6" t="inlineStr">
         <is>
-          <t>1차 매수선까지 20.0%</t>
+          <t>1차 매수선까지 16.1%</t>
         </is>
       </c>
       <c r="F50" s="7" t="n">
-        <v>55400</v>
+        <v>53700</v>
       </c>
       <c r="G50" s="7" t="n">
-        <v>55100</v>
+        <v>51500</v>
       </c>
       <c r="H50" s="7" t="n">
-        <v>57900</v>
+        <v>53700</v>
       </c>
       <c r="I50" s="7" t="n">
-        <v>57645</v>
+        <v>57735</v>
       </c>
       <c r="J50" s="7" t="n">
-        <v>46116</v>
+        <v>46188</v>
       </c>
       <c r="K50" s="7" t="n">
-        <v>46166</v>
+        <v>46238</v>
       </c>
       <c r="L50" s="8" t="n">
-        <v>0.2000173287700905</v>
+        <v>0.1613824127341148</v>
       </c>
       <c r="M50" s="9" t="inlineStr"/>
       <c r="N50" s="9" t="inlineStr"/>
       <c r="O50" s="7" t="n">
-        <v>41549.4</v>
+        <v>41614.2</v>
       </c>
       <c r="P50" s="8" t="n">
-        <v>0.3333525875223228</v>
+        <v>0.2904249030379052</v>
       </c>
       <c r="Q50" s="9" t="inlineStr"/>
       <c r="R50" s="9" t="inlineStr"/>
       <c r="S50" s="7" t="n">
-        <v>37394.46</v>
+        <v>37452.78000000001</v>
       </c>
       <c r="T50" s="8" t="n">
-        <v>0.4815028750248032</v>
+        <v>0.4338054478198946</v>
       </c>
       <c r="U50" s="9" t="inlineStr"/>
       <c r="V50" s="9" t="inlineStr"/>
@@ -4775,7 +4775,7 @@
       <c r="AD50" s="9" t="inlineStr"/>
       <c r="AE50" s="10" t="inlineStr">
         <is>
-          <t>2025-10-14 00:23:01</t>
+          <t>2025-10-16 03:37:19</t>
         </is>
       </c>
       <c r="AF50" s="11" t="n">
@@ -4807,45 +4807,45 @@
       </c>
       <c r="E51" s="6" t="inlineStr">
         <is>
-          <t>1차 매수선까지 20.4%</t>
+          <t>1차 매수선까지 24.0%</t>
         </is>
       </c>
       <c r="F51" s="7" t="n">
-        <v>28250</v>
+        <v>29050</v>
       </c>
       <c r="G51" s="7" t="n">
-        <v>27350</v>
+        <v>27950</v>
       </c>
       <c r="H51" s="7" t="n">
-        <v>28350</v>
+        <v>29200</v>
       </c>
       <c r="I51" s="7" t="n">
-        <v>29257.5</v>
+        <v>29227.5</v>
       </c>
       <c r="J51" s="7" t="n">
-        <v>23406</v>
+        <v>23382</v>
       </c>
       <c r="K51" s="7" t="n">
-        <v>23456</v>
+        <v>23432</v>
       </c>
       <c r="L51" s="8" t="n">
-        <v>0.2043826739427012</v>
+        <v>0.2397575964493001</v>
       </c>
       <c r="M51" s="9" t="inlineStr"/>
       <c r="N51" s="9" t="inlineStr"/>
       <c r="O51" s="7" t="n">
-        <v>21110.4</v>
+        <v>21088.8</v>
       </c>
       <c r="P51" s="8" t="n">
-        <v>0.3382029710474458</v>
+        <v>0.3775084404992224</v>
       </c>
       <c r="Q51" s="9" t="inlineStr"/>
       <c r="R51" s="9" t="inlineStr"/>
       <c r="S51" s="7" t="n">
-        <v>18999.36</v>
+        <v>18979.92</v>
       </c>
       <c r="T51" s="8" t="n">
-        <v>0.4868921900527175</v>
+        <v>0.5305649338880248</v>
       </c>
       <c r="U51" s="9" t="inlineStr"/>
       <c r="V51" s="9" t="inlineStr"/>
@@ -4859,7 +4859,7 @@
       <c r="AD51" s="9" t="inlineStr"/>
       <c r="AE51" s="10" t="inlineStr">
         <is>
-          <t>2025-10-14 00:23:02</t>
+          <t>2025-10-16 03:37:19</t>
         </is>
       </c>
       <c r="AF51" s="11" t="n">
@@ -4891,45 +4891,45 @@
       </c>
       <c r="E52" s="6" t="inlineStr">
         <is>
-          <t>1차 매수선까지 29.9%</t>
+          <t>1차 매수선까지 26.8%</t>
         </is>
       </c>
       <c r="F52" s="7" t="n">
-        <v>203500</v>
+        <v>200500</v>
       </c>
       <c r="G52" s="7" t="n">
-        <v>198500</v>
+        <v>195400</v>
       </c>
       <c r="H52" s="7" t="n">
-        <v>204500</v>
+        <v>201000</v>
       </c>
       <c r="I52" s="7" t="n">
-        <v>195190</v>
+        <v>196985</v>
       </c>
       <c r="J52" s="7" t="n">
-        <v>156152</v>
+        <v>157588</v>
       </c>
       <c r="K52" s="7" t="n">
-        <v>156652</v>
+        <v>158088</v>
       </c>
       <c r="L52" s="8" t="n">
-        <v>0.2990577841329827</v>
+        <v>0.2682809574414251</v>
       </c>
       <c r="M52" s="9" t="inlineStr"/>
       <c r="N52" s="9" t="inlineStr"/>
       <c r="O52" s="7" t="n">
-        <v>140986.8</v>
+        <v>142279.2</v>
       </c>
       <c r="P52" s="8" t="n">
-        <v>0.4433975379255361</v>
+        <v>0.4092010638238055</v>
       </c>
       <c r="Q52" s="9" t="inlineStr"/>
       <c r="R52" s="9" t="inlineStr"/>
       <c r="S52" s="7" t="n">
-        <v>126888.12</v>
+        <v>128051.28</v>
       </c>
       <c r="T52" s="8" t="n">
-        <v>0.6037750421394844</v>
+        <v>0.5657789598042283</v>
       </c>
       <c r="U52" s="9" t="inlineStr"/>
       <c r="V52" s="9" t="inlineStr"/>
@@ -4943,7 +4943,7 @@
       <c r="AD52" s="9" t="inlineStr"/>
       <c r="AE52" s="10" t="inlineStr">
         <is>
-          <t>2025-10-14 00:23:02</t>
+          <t>2025-10-16 03:37:20</t>
         </is>
       </c>
       <c r="AF52" s="11" t="n">
@@ -4975,45 +4975,45 @@
       </c>
       <c r="E53" s="6" t="inlineStr">
         <is>
-          <t>1차 매수선까지 19.5%</t>
+          <t>1차 매수선까지 16.9%</t>
         </is>
       </c>
       <c r="F53" s="7" t="n">
-        <v>54900</v>
+        <v>53100</v>
       </c>
       <c r="G53" s="7" t="n">
-        <v>53500</v>
+        <v>50800</v>
       </c>
       <c r="H53" s="7" t="n">
-        <v>55500</v>
+        <v>53200</v>
       </c>
       <c r="I53" s="7" t="n">
-        <v>57375</v>
+        <v>56705</v>
       </c>
       <c r="J53" s="7" t="n">
-        <v>45900</v>
+        <v>45364</v>
       </c>
       <c r="K53" s="7" t="n">
-        <v>45950</v>
+        <v>45414</v>
       </c>
       <c r="L53" s="8" t="n">
-        <v>0.1947769314472253</v>
+        <v>0.1692429647245343</v>
       </c>
       <c r="M53" s="9" t="inlineStr"/>
       <c r="N53" s="9" t="inlineStr"/>
       <c r="O53" s="7" t="n">
-        <v>41355</v>
+        <v>40872.6</v>
       </c>
       <c r="P53" s="8" t="n">
-        <v>0.3275299238302501</v>
+        <v>0.299158849693927</v>
       </c>
       <c r="Q53" s="9" t="inlineStr"/>
       <c r="R53" s="9" t="inlineStr"/>
       <c r="S53" s="7" t="n">
-        <v>37219.5</v>
+        <v>36785.34</v>
       </c>
       <c r="T53" s="8" t="n">
-        <v>0.4750332487002781</v>
+        <v>0.4435098329932524</v>
       </c>
       <c r="U53" s="9" t="inlineStr"/>
       <c r="V53" s="9" t="inlineStr"/>
@@ -5027,7 +5027,7 @@
       <c r="AD53" s="9" t="inlineStr"/>
       <c r="AE53" s="10" t="inlineStr">
         <is>
-          <t>2025-10-14 00:23:02</t>
+          <t>2025-10-16 03:37:20</t>
         </is>
       </c>
       <c r="AF53" s="11" t="n">
@@ -5059,45 +5059,45 @@
       </c>
       <c r="E54" s="6" t="inlineStr">
         <is>
-          <t>1차 매수선까지 16.8%</t>
+          <t>1차 매수선까지 22.4%</t>
         </is>
       </c>
       <c r="F54" s="7" t="n">
-        <v>14540</v>
+        <v>15200</v>
       </c>
       <c r="G54" s="7" t="n">
-        <v>14430</v>
+        <v>14450</v>
       </c>
       <c r="H54" s="7" t="n">
-        <v>15080</v>
+        <v>15270</v>
       </c>
       <c r="I54" s="7" t="n">
-        <v>15498</v>
+        <v>15455</v>
       </c>
       <c r="J54" s="7" t="n">
-        <v>12398.4</v>
+        <v>12364</v>
       </c>
       <c r="K54" s="7" t="n">
-        <v>12448.4</v>
+        <v>12414</v>
       </c>
       <c r="L54" s="8" t="n">
-        <v>0.1680215931364672</v>
+        <v>0.2244240373771548</v>
       </c>
       <c r="M54" s="9" t="inlineStr"/>
       <c r="N54" s="9" t="inlineStr"/>
       <c r="O54" s="7" t="n">
-        <v>11203.56</v>
+        <v>11172.6</v>
       </c>
       <c r="P54" s="8" t="n">
-        <v>0.2978017701516302</v>
+        <v>0.3604711526412831</v>
       </c>
       <c r="Q54" s="9" t="inlineStr"/>
       <c r="R54" s="9" t="inlineStr"/>
       <c r="S54" s="7" t="n">
-        <v>10083.204</v>
+        <v>10055.34</v>
       </c>
       <c r="T54" s="8" t="n">
-        <v>0.4420019668351446</v>
+        <v>0.5116346140458702</v>
       </c>
       <c r="U54" s="9" t="inlineStr"/>
       <c r="V54" s="9" t="inlineStr"/>
@@ -5111,7 +5111,7 @@
       <c r="AD54" s="9" t="inlineStr"/>
       <c r="AE54" s="10" t="inlineStr">
         <is>
-          <t>2025-10-14 00:23:03</t>
+          <t>2025-10-16 03:37:20</t>
         </is>
       </c>
       <c r="AF54" s="11" t="n">
@@ -5143,45 +5143,45 @@
       </c>
       <c r="E55" s="6" t="inlineStr">
         <is>
-          <t>1차 매수선까지 15.1%</t>
+          <t>1차 매수선까지 20.6%</t>
         </is>
       </c>
       <c r="F55" s="7" t="n">
-        <v>28650</v>
+        <v>29650</v>
       </c>
       <c r="G55" s="7" t="n">
-        <v>28200</v>
+        <v>28250</v>
       </c>
       <c r="H55" s="7" t="n">
-        <v>29050</v>
+        <v>29850</v>
       </c>
       <c r="I55" s="7" t="n">
-        <v>31057.5</v>
+        <v>30657.5</v>
       </c>
       <c r="J55" s="7" t="n">
-        <v>24846</v>
+        <v>24526</v>
       </c>
       <c r="K55" s="7" t="n">
-        <v>24896</v>
+        <v>24576</v>
       </c>
       <c r="L55" s="8" t="n">
-        <v>0.1507872750642673</v>
+        <v>0.2064615885416666</v>
       </c>
       <c r="M55" s="9" t="inlineStr"/>
       <c r="N55" s="9" t="inlineStr"/>
       <c r="O55" s="7" t="n">
-        <v>22406.4</v>
+        <v>22118.4</v>
       </c>
       <c r="P55" s="8" t="n">
-        <v>0.2786525278491859</v>
+        <v>0.3405128761574073</v>
       </c>
       <c r="Q55" s="9" t="inlineStr"/>
       <c r="R55" s="9" t="inlineStr"/>
       <c r="S55" s="7" t="n">
-        <v>20165.76</v>
+        <v>19906.56</v>
       </c>
       <c r="T55" s="8" t="n">
-        <v>0.4207250309435399</v>
+        <v>0.4894587512860081</v>
       </c>
       <c r="U55" s="9" t="inlineStr"/>
       <c r="V55" s="9" t="inlineStr"/>
@@ -5195,7 +5195,7 @@
       <c r="AD55" s="9" t="inlineStr"/>
       <c r="AE55" s="10" t="inlineStr">
         <is>
-          <t>2025-10-14 00:23:03</t>
+          <t>2025-10-16 03:37:21</t>
         </is>
       </c>
       <c r="AF55" s="11" t="n">
@@ -5227,45 +5227,45 @@
       </c>
       <c r="E56" s="6" t="inlineStr">
         <is>
-          <t>1차 매수선까지 13.8%</t>
+          <t>1차 매수선까지 18.9%</t>
         </is>
       </c>
       <c r="F56" s="7" t="n">
-        <v>2465</v>
+        <v>2545</v>
       </c>
       <c r="G56" s="7" t="n">
-        <v>2365</v>
+        <v>2440</v>
       </c>
       <c r="H56" s="7" t="n">
-        <v>2480</v>
+        <v>2562</v>
       </c>
       <c r="I56" s="7" t="n">
-        <v>2702.5</v>
+        <v>2669.25</v>
       </c>
       <c r="J56" s="7" t="n">
-        <v>2162</v>
+        <v>2135.4</v>
       </c>
       <c r="K56" s="7" t="n">
-        <v>2167</v>
+        <v>2140.4</v>
       </c>
       <c r="L56" s="8" t="n">
-        <v>0.1375173050299954</v>
+        <v>0.1890300878340496</v>
       </c>
       <c r="M56" s="9" t="inlineStr"/>
       <c r="N56" s="9" t="inlineStr"/>
       <c r="O56" s="7" t="n">
-        <v>1950.3</v>
+        <v>1926.36</v>
       </c>
       <c r="P56" s="8" t="n">
-        <v>0.2639081166999949</v>
+        <v>0.321144542037833</v>
       </c>
       <c r="Q56" s="9" t="inlineStr"/>
       <c r="R56" s="9" t="inlineStr"/>
       <c r="S56" s="7" t="n">
-        <v>1755.27</v>
+        <v>1733.724</v>
       </c>
       <c r="T56" s="8" t="n">
-        <v>0.4043423518888832</v>
+        <v>0.4679383800420365</v>
       </c>
       <c r="U56" s="9" t="inlineStr"/>
       <c r="V56" s="9" t="inlineStr"/>
@@ -5279,7 +5279,7 @@
       <c r="AD56" s="9" t="inlineStr"/>
       <c r="AE56" s="10" t="inlineStr">
         <is>
-          <t>2025-10-14 00:23:03</t>
+          <t>2025-10-16 03:37:21</t>
         </is>
       </c>
       <c r="AF56" s="11" t="n">
@@ -5306,50 +5306,50 @@
       </c>
       <c r="D57" s="5" t="inlineStr">
         <is>
-          <t>WATCHING</t>
+          <t>READY_BUY1</t>
         </is>
       </c>
       <c r="E57" s="6" t="inlineStr">
         <is>
-          <t>1차 매수선까지 13.2%</t>
+          <t>1차 매수선까지 6.8% (접근 중!)</t>
         </is>
       </c>
       <c r="F57" s="7" t="n">
-        <v>7410</v>
+        <v>6820</v>
       </c>
       <c r="G57" s="7" t="n">
-        <v>7220</v>
+        <v>6780</v>
       </c>
       <c r="H57" s="7" t="n">
-        <v>7670</v>
+        <v>7080</v>
       </c>
       <c r="I57" s="7" t="n">
-        <v>8171</v>
+        <v>7972.5</v>
       </c>
       <c r="J57" s="7" t="n">
-        <v>6536.8</v>
+        <v>6378</v>
       </c>
       <c r="K57" s="7" t="n">
-        <v>6546.8</v>
+        <v>6388</v>
       </c>
       <c r="L57" s="8" t="n">
-        <v>0.1318506751389992</v>
+        <v>0.06762680025046963</v>
       </c>
       <c r="M57" s="9" t="inlineStr"/>
       <c r="N57" s="9" t="inlineStr"/>
       <c r="O57" s="7" t="n">
-        <v>5892.12</v>
+        <v>5749.2</v>
       </c>
       <c r="P57" s="8" t="n">
-        <v>0.2576118612655547</v>
+        <v>0.1862520002782996</v>
       </c>
       <c r="Q57" s="9" t="inlineStr"/>
       <c r="R57" s="9" t="inlineStr"/>
       <c r="S57" s="7" t="n">
-        <v>5302.908</v>
+        <v>5174.28</v>
       </c>
       <c r="T57" s="8" t="n">
-        <v>0.3973465125172829</v>
+        <v>0.3180577780869996</v>
       </c>
       <c r="U57" s="9" t="inlineStr"/>
       <c r="V57" s="9" t="inlineStr"/>
@@ -5363,7 +5363,7 @@
       <c r="AD57" s="9" t="inlineStr"/>
       <c r="AE57" s="10" t="inlineStr">
         <is>
-          <t>2025-10-14 00:23:04</t>
+          <t>2025-10-16 03:37:21</t>
         </is>
       </c>
       <c r="AF57" s="11" t="n">
@@ -5395,45 +5395,45 @@
       </c>
       <c r="E58" s="6" t="inlineStr">
         <is>
-          <t>1차 매수선까지 40.0%</t>
+          <t>1차 매수선까지 49.5%</t>
         </is>
       </c>
       <c r="F58" s="7" t="n">
-        <v>157700</v>
+        <v>173400</v>
       </c>
       <c r="G58" s="7" t="n">
-        <v>143400</v>
+        <v>166100</v>
       </c>
       <c r="H58" s="7" t="n">
-        <v>160800</v>
+        <v>177700</v>
       </c>
       <c r="I58" s="7" t="n">
-        <v>140135</v>
+        <v>144320</v>
       </c>
       <c r="J58" s="7" t="n">
-        <v>112108</v>
+        <v>115456</v>
       </c>
       <c r="K58" s="7" t="n">
-        <v>112608</v>
+        <v>115956</v>
       </c>
       <c r="L58" s="8" t="n">
-        <v>0.4004333617504973</v>
+        <v>0.4953948049260064</v>
       </c>
       <c r="M58" s="9" t="inlineStr"/>
       <c r="N58" s="9" t="inlineStr"/>
       <c r="O58" s="7" t="n">
-        <v>101347.2</v>
+        <v>104360.4</v>
       </c>
       <c r="P58" s="8" t="n">
-        <v>0.5560370686116637</v>
+        <v>0.6615497832511181</v>
       </c>
       <c r="Q58" s="9" t="inlineStr"/>
       <c r="R58" s="9" t="inlineStr"/>
       <c r="S58" s="7" t="n">
-        <v>91212.48</v>
+        <v>93924.36000000002</v>
       </c>
       <c r="T58" s="8" t="n">
-        <v>0.7289300762351819</v>
+        <v>0.8461664258345756</v>
       </c>
       <c r="U58" s="9" t="inlineStr"/>
       <c r="V58" s="9" t="inlineStr"/>
@@ -5447,7 +5447,7 @@
       <c r="AD58" s="9" t="inlineStr"/>
       <c r="AE58" s="10" t="inlineStr">
         <is>
-          <t>2025-10-14 00:23:04</t>
+          <t>2025-10-16 03:37:22</t>
         </is>
       </c>
       <c r="AF58" s="11" t="n">
@@ -5479,45 +5479,45 @@
       </c>
       <c r="E59" s="6" t="inlineStr">
         <is>
-          <t>1차 매수선까지 25.2%</t>
+          <t>1차 매수선까지 20.4%</t>
         </is>
       </c>
       <c r="F59" s="7" t="n">
-        <v>151400</v>
+        <v>144900</v>
       </c>
       <c r="G59" s="7" t="n">
-        <v>147000</v>
+        <v>143000</v>
       </c>
       <c r="H59" s="7" t="n">
-        <v>158500</v>
+        <v>150200</v>
       </c>
       <c r="I59" s="7" t="n">
-        <v>150575</v>
+        <v>149835</v>
       </c>
       <c r="J59" s="7" t="n">
-        <v>120460</v>
+        <v>119868</v>
       </c>
       <c r="K59" s="7" t="n">
-        <v>120960</v>
+        <v>120368</v>
       </c>
       <c r="L59" s="8" t="n">
-        <v>0.2516534391534391</v>
+        <v>0.203808321148478</v>
       </c>
       <c r="M59" s="9" t="inlineStr"/>
       <c r="N59" s="9" t="inlineStr"/>
       <c r="O59" s="7" t="n">
-        <v>108864</v>
+        <v>108331.2</v>
       </c>
       <c r="P59" s="8" t="n">
-        <v>0.3907260435038213</v>
+        <v>0.3375648012760867</v>
       </c>
       <c r="Q59" s="9" t="inlineStr"/>
       <c r="R59" s="9" t="inlineStr"/>
       <c r="S59" s="7" t="n">
-        <v>97977.60000000001</v>
+        <v>97498.08</v>
       </c>
       <c r="T59" s="8" t="n">
-        <v>0.5452511594486901</v>
+        <v>0.4861831125289851</v>
       </c>
       <c r="U59" s="9" t="inlineStr"/>
       <c r="V59" s="9" t="inlineStr"/>
@@ -5531,7 +5531,7 @@
       <c r="AD59" s="9" t="inlineStr"/>
       <c r="AE59" s="10" t="inlineStr">
         <is>
-          <t>2025-10-14 00:23:04</t>
+          <t>2025-10-16 03:37:22</t>
         </is>
       </c>
       <c r="AF59" s="11" t="n">
@@ -5563,45 +5563,45 @@
       </c>
       <c r="E60" s="6" t="inlineStr">
         <is>
-          <t>1차 매수선까지 21.6%</t>
+          <t>1차 매수선까지 28.1%</t>
         </is>
       </c>
       <c r="F60" s="7" t="n">
-        <v>37150</v>
+        <v>39300</v>
       </c>
       <c r="G60" s="7" t="n">
-        <v>36800</v>
+        <v>38500</v>
       </c>
       <c r="H60" s="7" t="n">
-        <v>37850</v>
+        <v>41300</v>
       </c>
       <c r="I60" s="7" t="n">
-        <v>38115</v>
+        <v>38297.5</v>
       </c>
       <c r="J60" s="7" t="n">
-        <v>30492</v>
+        <v>30638</v>
       </c>
       <c r="K60" s="7" t="n">
-        <v>30542</v>
+        <v>30688</v>
       </c>
       <c r="L60" s="8" t="n">
-        <v>0.2163578023705062</v>
+        <v>0.2806308654848801</v>
       </c>
       <c r="M60" s="9" t="inlineStr"/>
       <c r="N60" s="9" t="inlineStr"/>
       <c r="O60" s="7" t="n">
-        <v>27487.8</v>
+        <v>27619.2</v>
       </c>
       <c r="P60" s="8" t="n">
-        <v>0.3515086693005625</v>
+        <v>0.4229231838720889</v>
       </c>
       <c r="Q60" s="9" t="inlineStr"/>
       <c r="R60" s="9" t="inlineStr"/>
       <c r="S60" s="7" t="n">
-        <v>24739.02</v>
+        <v>24857.28</v>
       </c>
       <c r="T60" s="8" t="n">
-        <v>0.5016762992228471</v>
+        <v>0.5810257598578765</v>
       </c>
       <c r="U60" s="9" t="inlineStr"/>
       <c r="V60" s="9" t="inlineStr"/>
@@ -5615,7 +5615,7 @@
       <c r="AD60" s="9" t="inlineStr"/>
       <c r="AE60" s="10" t="inlineStr">
         <is>
-          <t>2025-10-14 00:23:05</t>
+          <t>2025-10-16 03:37:22</t>
         </is>
       </c>
       <c r="AF60" s="11" t="n">
@@ -5642,50 +5642,50 @@
       </c>
       <c r="D61" s="5" t="inlineStr">
         <is>
-          <t>READY_BUY1</t>
+          <t>WATCHING</t>
         </is>
       </c>
       <c r="E61" s="6" t="inlineStr">
         <is>
-          <t>1차 매수선까지 9.2% (접근 중!)</t>
+          <t>1차 매수선까지 10.7%</t>
         </is>
       </c>
       <c r="F61" s="7" t="n">
-        <v>10220</v>
+        <v>10100</v>
       </c>
       <c r="G61" s="7" t="n">
-        <v>10050</v>
+        <v>9730</v>
       </c>
       <c r="H61" s="7" t="n">
-        <v>10540</v>
+        <v>10170</v>
       </c>
       <c r="I61" s="7" t="n">
-        <v>11685.5</v>
+        <v>11390.5</v>
       </c>
       <c r="J61" s="7" t="n">
-        <v>9348.4</v>
+        <v>9112.4</v>
       </c>
       <c r="K61" s="7" t="n">
-        <v>9358.4</v>
+        <v>9122.4</v>
       </c>
       <c r="L61" s="8" t="n">
-        <v>0.09206702000341943</v>
+        <v>0.1071647811979304</v>
       </c>
       <c r="M61" s="9" t="inlineStr"/>
       <c r="N61" s="9" t="inlineStr"/>
       <c r="O61" s="7" t="n">
-        <v>8422.559999999999</v>
+        <v>8210.16</v>
       </c>
       <c r="P61" s="8" t="n">
-        <v>0.2134078000037994</v>
+        <v>0.2301830902199226</v>
       </c>
       <c r="Q61" s="9" t="inlineStr"/>
       <c r="R61" s="9" t="inlineStr"/>
       <c r="S61" s="7" t="n">
-        <v>7580.304</v>
+        <v>7389.144</v>
       </c>
       <c r="T61" s="8" t="n">
-        <v>0.3482308888931103</v>
+        <v>0.3668701002443584</v>
       </c>
       <c r="U61" s="9" t="inlineStr"/>
       <c r="V61" s="9" t="inlineStr"/>
@@ -5699,7 +5699,7 @@
       <c r="AD61" s="9" t="inlineStr"/>
       <c r="AE61" s="10" t="inlineStr">
         <is>
-          <t>2025-10-14 00:23:05</t>
+          <t>2025-10-16 03:37:22</t>
         </is>
       </c>
       <c r="AF61" s="11" t="n">
@@ -5731,45 +5731,45 @@
       </c>
       <c r="E62" s="6" t="inlineStr">
         <is>
-          <t>1차 매수선까지 47.7%</t>
+          <t>1차 매수선까지 43.7%</t>
         </is>
       </c>
       <c r="F62" s="7" t="n">
-        <v>245500</v>
+        <v>246500</v>
       </c>
       <c r="G62" s="7" t="n">
-        <v>235000</v>
+        <v>232000</v>
       </c>
       <c r="H62" s="7" t="n">
-        <v>249000</v>
+        <v>246500</v>
       </c>
       <c r="I62" s="7" t="n">
-        <v>207080</v>
+        <v>213860</v>
       </c>
       <c r="J62" s="7" t="n">
-        <v>165664</v>
+        <v>171088</v>
       </c>
       <c r="K62" s="7" t="n">
-        <v>166164</v>
+        <v>171588</v>
       </c>
       <c r="L62" s="8" t="n">
-        <v>0.4774560073180713</v>
+        <v>0.436580646665268</v>
       </c>
       <c r="M62" s="9" t="inlineStr"/>
       <c r="N62" s="9" t="inlineStr"/>
       <c r="O62" s="7" t="n">
-        <v>149547.6</v>
+        <v>154429.2</v>
       </c>
       <c r="P62" s="8" t="n">
-        <v>0.641617785908968</v>
+        <v>0.5962007185169643</v>
       </c>
       <c r="Q62" s="9" t="inlineStr"/>
       <c r="R62" s="9" t="inlineStr"/>
       <c r="S62" s="7" t="n">
-        <v>134592.84</v>
+        <v>138986.28</v>
       </c>
       <c r="T62" s="8" t="n">
-        <v>0.8240197621210757</v>
+        <v>0.7735563539077378</v>
       </c>
       <c r="U62" s="9" t="inlineStr"/>
       <c r="V62" s="9" t="inlineStr"/>
@@ -5783,7 +5783,7 @@
       <c r="AD62" s="9" t="inlineStr"/>
       <c r="AE62" s="10" t="inlineStr">
         <is>
-          <t>2025-10-14 00:23:05</t>
+          <t>2025-10-16 03:37:23</t>
         </is>
       </c>
       <c r="AF62" s="11" t="n">
@@ -5815,45 +5815,45 @@
       </c>
       <c r="E63" s="6" t="inlineStr">
         <is>
-          <t>1차 매수선까지 21.8%</t>
+          <t>1차 매수선까지 24.8%</t>
         </is>
       </c>
       <c r="F63" s="7" t="n">
-        <v>272500</v>
+        <v>279000</v>
       </c>
       <c r="G63" s="7" t="n">
-        <v>259500</v>
+        <v>275000</v>
       </c>
       <c r="H63" s="7" t="n">
-        <v>273000</v>
+        <v>279500</v>
       </c>
       <c r="I63" s="7" t="n">
-        <v>279100</v>
+        <v>278925</v>
       </c>
       <c r="J63" s="7" t="n">
-        <v>223280</v>
+        <v>223140</v>
       </c>
       <c r="K63" s="7" t="n">
-        <v>223780</v>
+        <v>223640</v>
       </c>
       <c r="L63" s="8" t="n">
-        <v>0.2177138260791849</v>
+        <v>0.2475406903952781</v>
       </c>
       <c r="M63" s="9" t="inlineStr"/>
       <c r="N63" s="9" t="inlineStr"/>
       <c r="O63" s="7" t="n">
-        <v>201402</v>
+        <v>201276</v>
       </c>
       <c r="P63" s="8" t="n">
-        <v>0.3530153623102055</v>
+        <v>0.3861563226614201</v>
       </c>
       <c r="Q63" s="9" t="inlineStr"/>
       <c r="R63" s="9" t="inlineStr"/>
       <c r="S63" s="7" t="n">
-        <v>181261.8</v>
+        <v>181148.4</v>
       </c>
       <c r="T63" s="8" t="n">
-        <v>0.5033504025668948</v>
+        <v>0.5401736918460224</v>
       </c>
       <c r="U63" s="9" t="inlineStr"/>
       <c r="V63" s="9" t="inlineStr"/>
@@ -5867,7 +5867,7 @@
       <c r="AD63" s="9" t="inlineStr"/>
       <c r="AE63" s="10" t="inlineStr">
         <is>
-          <t>2025-10-14 00:23:06</t>
+          <t>2025-10-16 03:37:23</t>
         </is>
       </c>
       <c r="AF63" s="11" t="n">
@@ -5899,45 +5899,45 @@
       </c>
       <c r="E64" s="6" t="inlineStr">
         <is>
-          <t>1차 매수선까지 20.5%</t>
+          <t>1차 매수선까지 24.7%</t>
         </is>
       </c>
       <c r="F64" s="7" t="n">
-        <v>92200</v>
+        <v>95300</v>
       </c>
       <c r="G64" s="7" t="n">
-        <v>91600</v>
+        <v>92000</v>
       </c>
       <c r="H64" s="7" t="n">
-        <v>96000</v>
+        <v>96400</v>
       </c>
       <c r="I64" s="7" t="n">
-        <v>95530</v>
+        <v>95380</v>
       </c>
       <c r="J64" s="7" t="n">
-        <v>76424</v>
+        <v>76304</v>
       </c>
       <c r="K64" s="7" t="n">
-        <v>76524</v>
+        <v>76404</v>
       </c>
       <c r="L64" s="8" t="n">
-        <v>0.2048507657728294</v>
+        <v>0.2473168944034344</v>
       </c>
       <c r="M64" s="9" t="inlineStr"/>
       <c r="N64" s="9" t="inlineStr"/>
       <c r="O64" s="7" t="n">
-        <v>68871.60000000001</v>
+        <v>68763.60000000001</v>
       </c>
       <c r="P64" s="8" t="n">
-        <v>0.3387230730809215</v>
+        <v>0.3859076604482603</v>
       </c>
       <c r="Q64" s="9" t="inlineStr"/>
       <c r="R64" s="9" t="inlineStr"/>
       <c r="S64" s="7" t="n">
-        <v>61984.44000000001</v>
+        <v>61887.24000000001</v>
       </c>
       <c r="T64" s="8" t="n">
-        <v>0.4874700812010238</v>
+        <v>0.539897400498067</v>
       </c>
       <c r="U64" s="9" t="inlineStr"/>
       <c r="V64" s="9" t="inlineStr"/>
@@ -5951,7 +5951,7 @@
       <c r="AD64" s="9" t="inlineStr"/>
       <c r="AE64" s="10" t="inlineStr">
         <is>
-          <t>2025-10-14 00:23:06</t>
+          <t>2025-10-16 03:37:23</t>
         </is>
       </c>
       <c r="AF64" s="11" t="n">
@@ -5983,45 +5983,45 @@
       </c>
       <c r="E65" s="6" t="inlineStr">
         <is>
-          <t>1차 매수선까지 19.7%</t>
+          <t>1차 매수선까지 19.4%</t>
         </is>
       </c>
       <c r="F65" s="7" t="n">
-        <v>84000</v>
+        <v>83400</v>
       </c>
       <c r="G65" s="7" t="n">
-        <v>81200</v>
+        <v>79700</v>
       </c>
       <c r="H65" s="7" t="n">
-        <v>84100</v>
+        <v>83500</v>
       </c>
       <c r="I65" s="7" t="n">
-        <v>87565</v>
+        <v>87175</v>
       </c>
       <c r="J65" s="7" t="n">
-        <v>70052</v>
+        <v>69740</v>
       </c>
       <c r="K65" s="7" t="n">
-        <v>70152</v>
+        <v>69840</v>
       </c>
       <c r="L65" s="8" t="n">
-        <v>0.1973999315771468</v>
+        <v>0.1941580756013746</v>
       </c>
       <c r="M65" s="9" t="inlineStr"/>
       <c r="N65" s="9" t="inlineStr"/>
       <c r="O65" s="7" t="n">
-        <v>63136.8</v>
+        <v>62856</v>
       </c>
       <c r="P65" s="8" t="n">
-        <v>0.3304443684190519</v>
+        <v>0.3268423062237495</v>
       </c>
       <c r="Q65" s="9" t="inlineStr"/>
       <c r="R65" s="9" t="inlineStr"/>
       <c r="S65" s="7" t="n">
-        <v>56823.12</v>
+        <v>56570.4</v>
       </c>
       <c r="T65" s="8" t="n">
-        <v>0.4782715204656132</v>
+        <v>0.4742692291374994</v>
       </c>
       <c r="U65" s="9" t="inlineStr"/>
       <c r="V65" s="9" t="inlineStr"/>
@@ -6035,7 +6035,7 @@
       <c r="AD65" s="9" t="inlineStr"/>
       <c r="AE65" s="10" t="inlineStr">
         <is>
-          <t>2025-10-14 00:23:07</t>
+          <t>2025-10-16 03:37:23</t>
         </is>
       </c>
       <c r="AF65" s="11" t="n">
@@ -6067,45 +6067,45 @@
       </c>
       <c r="E66" s="6" t="inlineStr">
         <is>
-          <t>1차 매수선까지 25.6%</t>
+          <t>1차 매수선까지 32.3%</t>
         </is>
       </c>
       <c r="F66" s="7" t="n">
-        <v>222000</v>
+        <v>234500</v>
       </c>
       <c r="G66" s="7" t="n">
-        <v>216500</v>
+        <v>221000</v>
       </c>
       <c r="H66" s="7" t="n">
-        <v>228000</v>
+        <v>236000</v>
       </c>
       <c r="I66" s="7" t="n">
-        <v>220275</v>
+        <v>220925</v>
       </c>
       <c r="J66" s="7" t="n">
-        <v>176220</v>
+        <v>176740</v>
       </c>
       <c r="K66" s="7" t="n">
-        <v>176720</v>
+        <v>177240</v>
       </c>
       <c r="L66" s="8" t="n">
-        <v>0.2562245359891354</v>
+        <v>0.3230647709320695</v>
       </c>
       <c r="M66" s="9" t="inlineStr"/>
       <c r="N66" s="9" t="inlineStr"/>
       <c r="O66" s="7" t="n">
-        <v>159048</v>
+        <v>159516</v>
       </c>
       <c r="P66" s="8" t="n">
-        <v>0.395805039987928</v>
+        <v>0.4700719677022995</v>
       </c>
       <c r="Q66" s="9" t="inlineStr"/>
       <c r="R66" s="9" t="inlineStr"/>
       <c r="S66" s="7" t="n">
-        <v>143143.2</v>
+        <v>143564.4</v>
       </c>
       <c r="T66" s="8" t="n">
-        <v>0.5508944888754757</v>
+        <v>0.6334132974469995</v>
       </c>
       <c r="U66" s="9" t="inlineStr"/>
       <c r="V66" s="9" t="inlineStr"/>
@@ -6119,7 +6119,7 @@
       <c r="AD66" s="9" t="inlineStr"/>
       <c r="AE66" s="10" t="inlineStr">
         <is>
-          <t>2025-10-14 00:23:07</t>
+          <t>2025-10-16 03:37:24</t>
         </is>
       </c>
       <c r="AF66" s="11" t="n">
@@ -6151,45 +6151,45 @@
       </c>
       <c r="E67" s="6" t="inlineStr">
         <is>
-          <t>1차 매수선까지 24.4%</t>
+          <t>1차 매수선까지 28.7%</t>
         </is>
       </c>
       <c r="F67" s="7" t="n">
-        <v>104000</v>
+        <v>107700</v>
       </c>
       <c r="G67" s="7" t="n">
-        <v>100300</v>
+        <v>106000</v>
       </c>
       <c r="H67" s="7" t="n">
-        <v>104400</v>
+        <v>107800</v>
       </c>
       <c r="I67" s="7" t="n">
-        <v>104360</v>
+        <v>104485</v>
       </c>
       <c r="J67" s="7" t="n">
-        <v>83488</v>
+        <v>83588</v>
       </c>
       <c r="K67" s="7" t="n">
-        <v>83588</v>
+        <v>83688</v>
       </c>
       <c r="L67" s="8" t="n">
-        <v>0.2441977317318275</v>
+        <v>0.2869228563234872</v>
       </c>
       <c r="M67" s="9" t="inlineStr"/>
       <c r="N67" s="9" t="inlineStr"/>
       <c r="O67" s="7" t="n">
-        <v>75229.2</v>
+        <v>75319.2</v>
       </c>
       <c r="P67" s="8" t="n">
-        <v>0.3824419241464751</v>
+        <v>0.4299142848038748</v>
       </c>
       <c r="Q67" s="9" t="inlineStr"/>
       <c r="R67" s="9" t="inlineStr"/>
       <c r="S67" s="7" t="n">
-        <v>67706.28</v>
+        <v>67787.28</v>
       </c>
       <c r="T67" s="8" t="n">
-        <v>0.5360465823849723</v>
+        <v>0.588793649782083</v>
       </c>
       <c r="U67" s="9" t="inlineStr"/>
       <c r="V67" s="9" t="inlineStr"/>
@@ -6203,7 +6203,7 @@
       <c r="AD67" s="9" t="inlineStr"/>
       <c r="AE67" s="10" t="inlineStr">
         <is>
-          <t>2025-10-14 00:23:07</t>
+          <t>2025-10-16 03:37:24</t>
         </is>
       </c>
       <c r="AF67" s="11" t="n">
@@ -6211,6 +6211,90 @@
       </c>
       <c r="AG67" s="6" t="inlineStr"/>
       <c r="AH67" s="6" t="inlineStr"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="5" t="inlineStr">
+        <is>
+          <t>0008Z0</t>
+        </is>
+      </c>
+      <c r="B68" s="5" t="inlineStr">
+        <is>
+          <t>에스엔시스</t>
+        </is>
+      </c>
+      <c r="C68" s="5" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="D68" s="5" t="inlineStr">
+        <is>
+          <t>WATCHING</t>
+        </is>
+      </c>
+      <c r="E68" s="6" t="inlineStr">
+        <is>
+          <t>1차 매수선까지 13.5%</t>
+        </is>
+      </c>
+      <c r="F68" s="7" t="n">
+        <v>38900</v>
+      </c>
+      <c r="G68" s="7" t="n">
+        <v>38600</v>
+      </c>
+      <c r="H68" s="7" t="n">
+        <v>40800</v>
+      </c>
+      <c r="I68" s="7" t="n">
+        <v>42782.5</v>
+      </c>
+      <c r="J68" s="7" t="n">
+        <v>34226</v>
+      </c>
+      <c r="K68" s="7" t="n">
+        <v>34276</v>
+      </c>
+      <c r="L68" s="8" t="n">
+        <v>1.349048897187536e-07</v>
+      </c>
+      <c r="M68" s="9" t="inlineStr"/>
+      <c r="N68" s="9" t="inlineStr"/>
+      <c r="O68" s="7" t="n">
+        <v>30848.4</v>
+      </c>
+      <c r="P68" s="8" t="n">
+        <v>2.610054330208374e-07</v>
+      </c>
+      <c r="Q68" s="9" t="inlineStr"/>
+      <c r="R68" s="9" t="inlineStr"/>
+      <c r="S68" s="7" t="n">
+        <v>27763.56</v>
+      </c>
+      <c r="T68" s="8" t="n">
+        <v>4.011171478009304e-07</v>
+      </c>
+      <c r="U68" s="9" t="inlineStr"/>
+      <c r="V68" s="9" t="inlineStr"/>
+      <c r="W68" s="9" t="inlineStr"/>
+      <c r="X68" s="9" t="inlineStr"/>
+      <c r="Y68" s="9" t="inlineStr"/>
+      <c r="Z68" s="9" t="inlineStr"/>
+      <c r="AA68" s="9" t="inlineStr"/>
+      <c r="AB68" s="9" t="inlineStr"/>
+      <c r="AC68" s="9" t="inlineStr"/>
+      <c r="AD68" s="9" t="inlineStr"/>
+      <c r="AE68" s="10" t="inlineStr">
+        <is>
+          <t>2025-10-14 22:40:06</t>
+        </is>
+      </c>
+      <c r="AF68" s="11" t="n">
+        <v>45888</v>
+      </c>
+      <c r="AG68" s="6" t="inlineStr"/>
+      <c r="AH68" s="6" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>